<commit_message>
Evidence/Gap up to 3rd Control
</commit_message>
<xml_diff>
--- a/compliance/Control_Matrix_Mapping.xlsx
+++ b/compliance/Control_Matrix_Mapping.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kate\OneDrive\Documents\GRC_Risk_Assessment\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kate\OneDrive\Documents\GRC_Risk_Assessment\C3-GRC\compliance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB6567A9-66BD-46BB-AA35-FA31CC6ECE67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0924E4B-59CB-4C8C-B5E1-0A817417CD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,25 @@
     <sheet name="Control Matrix Mapping" sheetId="1" r:id="rId1"/>
     <sheet name="CM Legend" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="240">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="241">
   <si>
     <t>CrochetCrochetCrochet (C3) — ISO 27001:2022 / NIST 800-53 Control Matrix</t>
   </si>
@@ -740,13 +753,16 @@
     <t>The process appears to be operationally managed through Rippling and Entra ID but without a documented runbook defining steps, timelines, or verification requirements for provisioning and deprovisioning.</t>
   </si>
   <si>
-    <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C</t>
-  </si>
-  <si>
     <t>Microsoft Entra ID [C3-013] serves as the primary identity provider for C3, issuing and managing identities across all SSO-connected SaaS platforms including Microsoft 365, GitHub, 1Password, and Rippling. Each employee holds a unique Employee ID (EMP-001 through EMP-016) with a corresponding Entra ID identity. Iris Cohen (People &amp; Operations Coordinator) administers Rippling [C3-024], which manages the employee lifecycle including onboarding and offboarding workflows. Iris is noted as responsible for onboarding/offboarding access provisioning. No formal identity lifecycle management procedure was identified.</t>
   </si>
   <si>
     <t>All 17 endpoints are enrolled in Microsoft Intune MDM (C3-010), providing a baseline device compliance and configuration management layer. Endpoint Detection and Response (EDR) is explicitly confirmed on three high-risk devices: Devon Nakamura's MacBook Pro (C3-EMP-003, Full AWS Admin), Jordan Ellis's MacBook Pro (C3-EMP-006, AWS Admin / IaC owner), and Sofia Reyes's MacBook Pro (C3-EMP-004, Senior Software Engineer). GitHub secret scanning (C3-008) is active to detect accidentally committed credentials. FileVault encryption is enabled on all macOS devices. EDR coverage is not confirmed for the remaining 14 endpoints, including all MacBook Air devices assigned to Customer Success, Marketing, Operations, and Content staff. No anti-malware or EDR solution is referenced for the standard employee device fleet. There is no evidence of a centrally managed anti-malware policy, coverage reporting, or defined response procedure for malware detection events.</t>
+  </si>
+  <si>
+    <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C3-013]. Privileged accounts are required to use hardware security keys for any admin account activity. All credentials are stored and managed by 1Password [C3-020], with vault segmentation by department, preventing cross-functional exposure. No formal password policy is defined. No recovery procedures are defined.</t>
+  </si>
+  <si>
+    <t>Technical controls are in place via 1Password, however there are no formal policies or procedures in place for password policy, requirements, rotation scheduling, etc.</t>
   </si>
 </sst>
 </file>
@@ -1538,9 +1554,9 @@
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.77734375" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="24.6640625" customWidth="1"/>
-    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="4" max="4" width="14" hidden="1" customWidth="1"/>
     <col min="5" max="5" width="16.33203125" customWidth="1"/>
     <col min="7" max="7" width="45.33203125" customWidth="1"/>
     <col min="8" max="8" width="10.77734375" customWidth="1"/>
@@ -1816,7 +1832,7 @@
         <v>228</v>
       </c>
       <c r="L6" s="59" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="M6" s="10" t="s">
         <v>236</v>
@@ -1835,7 +1851,7 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>48</v>
       </c>
@@ -1866,9 +1882,11 @@
         <v>227</v>
       </c>
       <c r="L7" s="58" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
-      <c r="M7" s="7"/>
+      <c r="M7" s="7" t="s">
+        <v>240</v>
+      </c>
       <c r="N7" s="7"/>
       <c r="O7" s="8"/>
       <c r="P7" s="1"/>
@@ -2374,7 +2392,7 @@
         <v>231</v>
       </c>
       <c r="L18" s="58" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>

</xml_diff>

<commit_message>
Control 4, Clean Up
</commit_message>
<xml_diff>
--- a/compliance/Control_Matrix_Mapping.xlsx
+++ b/compliance/Control_Matrix_Mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kate\OneDrive\Documents\GRC_Risk_Assessment\C3-GRC\compliance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0924E4B-59CB-4C8C-B5E1-0A817417CD7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D0E0E3-B670-419B-A70C-49BF91B21524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="242">
   <si>
     <t>CrochetCrochetCrochet (C3) — ISO 27001:2022 / NIST 800-53 Control Matrix</t>
   </si>
@@ -744,9 +744,6 @@
     <t>Need SDLC offical documentation; Need additional security testing</t>
   </si>
   <si>
-    <t>Role-based access control in implemented and operationally enforced through Microsoft Entra ID Conditional Access rules, [C3-013]. This governs authentication and device compliance requirements for all SaaS and cloud environment access. 1Password Teams  [C3-020) vaults are segmented by department, with credential access limited by function. Employee system access is provisioned per role. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts. No formal policy is identified or referenced.</t>
-  </si>
-  <si>
     <t xml:space="preserve">The control is operationally practiced, but not formally documented or communicated as a policy artifact. </t>
   </si>
   <si>
@@ -756,13 +753,19 @@
     <t>Microsoft Entra ID [C3-013] serves as the primary identity provider for C3, issuing and managing identities across all SSO-connected SaaS platforms including Microsoft 365, GitHub, 1Password, and Rippling. Each employee holds a unique Employee ID (EMP-001 through EMP-016) with a corresponding Entra ID identity. Iris Cohen (People &amp; Operations Coordinator) administers Rippling [C3-024], which manages the employee lifecycle including onboarding and offboarding workflows. Iris is noted as responsible for onboarding/offboarding access provisioning. No formal identity lifecycle management procedure was identified.</t>
   </si>
   <si>
-    <t>All 17 endpoints are enrolled in Microsoft Intune MDM (C3-010), providing a baseline device compliance and configuration management layer. Endpoint Detection and Response (EDR) is explicitly confirmed on three high-risk devices: Devon Nakamura's MacBook Pro (C3-EMP-003, Full AWS Admin), Jordan Ellis's MacBook Pro (C3-EMP-006, AWS Admin / IaC owner), and Sofia Reyes's MacBook Pro (C3-EMP-004, Senior Software Engineer). GitHub secret scanning (C3-008) is active to detect accidentally committed credentials. FileVault encryption is enabled on all macOS devices. EDR coverage is not confirmed for the remaining 14 endpoints, including all MacBook Air devices assigned to Customer Success, Marketing, Operations, and Content staff. No anti-malware or EDR solution is referenced for the standard employee device fleet. There is no evidence of a centrally managed anti-malware policy, coverage reporting, or defined response procedure for malware detection events.</t>
-  </si>
-  <si>
     <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C3-013]. Privileged accounts are required to use hardware security keys for any admin account activity. All credentials are stored and managed by 1Password [C3-020], with vault segmentation by department, preventing cross-functional exposure. No formal password policy is defined. No recovery procedures are defined.</t>
   </si>
   <si>
     <t>Technical controls are in place via 1Password, however there are no formal policies or procedures in place for password policy, requirements, rotation scheduling, etc.</t>
+  </si>
+  <si>
+    <t>Role-based access control in implemented and operationally enforced through Microsoft Entra ID Conditional Access rules, [C3-013]. This governs authentication and device compliance requirements for all SaaS and cloud environment access. 1Password Teams  [C3-020] vaults are segmented by department, with credential access limited by function. Employee system access is provisioned per role. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts. No formal policy is identified or referenced.</t>
+  </si>
+  <si>
+    <t>Access provisioning follows the least-privilege model, by role-differentiated system access. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts.  1Password [C3-020] vault segmentation enforces access boundaries by department. No formal access rights review is documented, no procedures for access rights are documented.</t>
+  </si>
+  <si>
+    <t>Technical contros are in place via 1Password, however, no formal access rights review schedule, documented provisioning and deprovisioning procedures, or periodic recertification process have been identified beyond the noted quarterly review for privileged accounts.</t>
   </si>
 </sst>
 </file>
@@ -1782,10 +1785,10 @@
         <v>227</v>
       </c>
       <c r="L5" s="58" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="M5" s="7" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="8"/>
@@ -1832,10 +1835,10 @@
         <v>228</v>
       </c>
       <c r="L6" s="59" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="M6" s="10" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="N6" s="10"/>
       <c r="O6" s="11"/>
@@ -1882,10 +1885,10 @@
         <v>227</v>
       </c>
       <c r="L7" s="58" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="8"/>
@@ -1901,7 +1904,7 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>54</v>
       </c>
@@ -1931,8 +1934,12 @@
       <c r="K8" s="59" t="s">
         <v>227</v>
       </c>
-      <c r="L8" s="59"/>
-      <c r="M8" s="10"/>
+      <c r="L8" s="59" t="s">
+        <v>240</v>
+      </c>
+      <c r="M8" s="10" t="s">
+        <v>241</v>
+      </c>
       <c r="N8" s="10"/>
       <c r="O8" s="11"/>
       <c r="P8" s="1"/>
@@ -2361,7 +2368,7 @@
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
     </row>
-    <row r="18" spans="1:26" ht="273.60000000000002" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="22.8" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>119</v>
       </c>
@@ -2391,9 +2398,7 @@
       <c r="K18" s="58" t="s">
         <v>231</v>
       </c>
-      <c r="L18" s="58" t="s">
-        <v>238</v>
-      </c>
+      <c r="L18" s="58"/>
       <c r="M18" s="7"/>
       <c r="N18" s="7"/>
       <c r="O18" s="8"/>

</xml_diff>

<commit_message>
Catching up w/ imp. & maturity scoring
</commit_message>
<xml_diff>
--- a/compliance/Control_Matrix_Mapping.xlsx
+++ b/compliance/Control_Matrix_Mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kate\OneDrive\Documents\GRC_Risk_Assessment\C3-GRC\compliance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6D0E0E3-B670-419B-A70C-49BF91B21524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E81B5988-A7B6-4DBB-983C-453667F224B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="308" uniqueCount="243">
   <si>
     <t>CrochetCrochetCrochet (C3) — ISO 27001:2022 / NIST 800-53 Control Matrix</t>
   </si>
@@ -766,6 +766,9 @@
   </si>
   <si>
     <t>Technical contros are in place via 1Password, however, no formal access rights review schedule, documented provisioning and deprovisioning procedures, or periodic recertification process have been identified beyond the noted quarterly review for privileged accounts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Partial </t>
   </si>
 </sst>
 </file>
@@ -1829,8 +1832,12 @@
       <c r="H6" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I6" s="11"/>
-      <c r="J6" s="12"/>
+      <c r="I6" s="11" t="s">
+        <v>242</v>
+      </c>
+      <c r="J6" s="12">
+        <v>2</v>
+      </c>
       <c r="K6" s="59" t="s">
         <v>228</v>
       </c>
@@ -1879,8 +1886,12 @@
       <c r="H7" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I7" s="8"/>
-      <c r="J7" s="9"/>
+      <c r="I7" s="8" t="s">
+        <v>242</v>
+      </c>
+      <c r="J7" s="9">
+        <v>2</v>
+      </c>
       <c r="K7" s="58" t="s">
         <v>227</v>
       </c>
@@ -1929,8 +1940,12 @@
       <c r="H8" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I8" s="11"/>
-      <c r="J8" s="12"/>
+      <c r="I8" s="11" t="s">
+        <v>198</v>
+      </c>
+      <c r="J8" s="12">
+        <v>2</v>
+      </c>
       <c r="K8" s="59" t="s">
         <v>227</v>
       </c>

</xml_diff>

<commit_message>
Took a break, back for 8&9
</commit_message>
<xml_diff>
--- a/compliance/Control_Matrix_Mapping.xlsx
+++ b/compliance/Control_Matrix_Mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kate\OneDrive\Documents\GRC_Risk_Assessment\C3-GRC\compliance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC83B5E2-F787-4B79-AE38-0F6A4CD940C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7090FAC3-5360-41A7-881D-61549FAE4AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="254">
   <si>
     <t>CrochetCrochetCrochet (C3) — ISO 27001:2022 / NIST 800-53 Control Matrix</t>
   </si>
@@ -788,6 +788,21 @@
   <si>
     <t xml:space="preserve">Missing </t>
   </si>
+  <si>
+    <t>No formal Information Security Policy document has been identified in the asset inventory, employee directory, or any referenced system notes. Security controls are operationally implemented across the environmen and ownership is assigned per control in this matrix. However, there is no evidence of a management-approved, published, and communicated information security policy that establishes C3's security intent, objectives, or responsibilities. The absence of this foundational document means all other controls lack a governing policy framework to reference, which represents a significant gap for any ISO 27001 audit.</t>
+  </si>
+  <si>
+    <t>Completely missing.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Regulatory awareness appears operationally embedded but not formally catalogued or reviewed on a defined schedule.</t>
+  </si>
+  <si>
+    <t>PII is identified and flagged across the entire asset inventory using a dedicated 'Contains PII' column applied to all 42 assets. No formal Privacy Policy or PII handling procedure document has been identified. There is no documented process for responding to data subject access requests or right-to-erasure requests, which is a meaningful gap given C3's customer PII exposure and GDPR-adjacent obligations.</t>
+  </si>
+  <si>
+    <t>C3 operates in a regulatory environment touching multiple frameworks. PCI DSS obligations arise from subscription payment processing via Stripe [C3-012]; C3 mitigates direct PCI scope by tokenizing all payment card data through Stripe rather than storing raw card data. ISO 27001 compliance tags are applied to all 42 assets in the asset inventory. Customer PII and employee PII are present across multiple assets [C3-001, C3-002, C3-004, C3-015, C3-024], indicating GDPR and applicable U.S. privacy law obligations. Marcus Okafor is noted as responsible for finance and compliance-adjacent functions. No formal legal and regulatory register has been identified documenting all applicable obligations, their sources, review dates, or responsible owners</t>
+  </si>
 </sst>
 </file>
 
@@ -1187,7 +1202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="73">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1339,11 +1354,18 @@
     <xf numFmtId="0" fontId="26" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -1356,14 +1378,14 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1586,36 +1608,39 @@
   <dimension ref="A1:Z995"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.77734375" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" customWidth="1"/>
-    <col min="4" max="4" width="14" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" customWidth="1"/>
-    <col min="7" max="7" width="45.33203125" customWidth="1"/>
-    <col min="8" max="8" width="10.77734375" customWidth="1"/>
-    <col min="12" max="12" width="33.88671875" customWidth="1"/>
-    <col min="13" max="13" width="28.109375" customWidth="1"/>
-    <col min="14" max="14" width="24.33203125" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" style="73" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" style="73" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" style="73" customWidth="1"/>
+    <col min="4" max="4" width="14" style="73" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" style="73" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" style="73"/>
+    <col min="7" max="7" width="45.33203125" style="73" customWidth="1"/>
+    <col min="8" max="8" width="10.77734375" style="73" customWidth="1"/>
+    <col min="9" max="11" width="12.6640625" style="73"/>
+    <col min="12" max="12" width="33.88671875" style="73" customWidth="1"/>
+    <col min="13" max="13" width="28.109375" style="73" customWidth="1"/>
+    <col min="14" max="14" width="24.33203125" style="73" customWidth="1"/>
+    <col min="15" max="16384" width="12.6640625" style="73"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="63" t="s">
+      <c r="A1" s="66" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
-      <c r="F1" s="64"/>
-      <c r="G1" s="64"/>
-      <c r="H1" s="64"/>
-      <c r="I1" s="64"/>
-      <c r="J1" s="64"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="64"/>
-      <c r="N1" s="64"/>
-      <c r="O1" s="65"/>
+      <c r="B1" s="71"/>
+      <c r="C1" s="71"/>
+      <c r="D1" s="71"/>
+      <c r="E1" s="71"/>
+      <c r="F1" s="71"/>
+      <c r="G1" s="71"/>
+      <c r="H1" s="71"/>
+      <c r="I1" s="71"/>
+      <c r="J1" s="71"/>
+      <c r="K1" s="71"/>
+      <c r="L1" s="71"/>
+      <c r="M1" s="71"/>
+      <c r="N1" s="71"/>
+      <c r="O1" s="72"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -1629,29 +1654,29 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="21" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="66" t="s">
+      <c r="A2" s="67" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="64"/>
-      <c r="C2" s="64"/>
-      <c r="D2" s="64"/>
-      <c r="E2" s="65"/>
-      <c r="F2" s="67" t="s">
+      <c r="B2" s="71"/>
+      <c r="C2" s="71"/>
+      <c r="D2" s="71"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="65"/>
-      <c r="H2" s="68" t="s">
+      <c r="G2" s="72"/>
+      <c r="H2" s="69" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="64"/>
-      <c r="J2" s="64"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="65"/>
-      <c r="M2" s="69" t="s">
+      <c r="I2" s="71"/>
+      <c r="J2" s="71"/>
+      <c r="K2" s="71"/>
+      <c r="L2" s="72"/>
+      <c r="M2" s="70" t="s">
         <v>4</v>
       </c>
-      <c r="N2" s="64"/>
-      <c r="O2" s="65"/>
+      <c r="N2" s="71"/>
+      <c r="O2" s="72"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -2077,7 +2102,7 @@
       <c r="H10" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I10" s="72" t="s">
+      <c r="I10" s="65" t="s">
         <v>198</v>
       </c>
       <c r="J10" s="12">
@@ -2086,10 +2111,10 @@
       <c r="K10" s="59" t="s">
         <v>227</v>
       </c>
-      <c r="L10" s="70" t="s">
+      <c r="L10" s="63" t="s">
         <v>246</v>
       </c>
-      <c r="M10" s="71" t="s">
+      <c r="M10" s="64" t="s">
         <v>247</v>
       </c>
       <c r="N10" s="10"/>
@@ -2106,7 +2131,7 @@
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" ht="182.4" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>72</v>
       </c>
@@ -2140,8 +2165,12 @@
       <c r="K11" s="58" t="s">
         <v>229</v>
       </c>
-      <c r="L11" s="58"/>
-      <c r="M11" s="7"/>
+      <c r="L11" s="58" t="s">
+        <v>249</v>
+      </c>
+      <c r="M11" s="7" t="s">
+        <v>250</v>
+      </c>
       <c r="N11" s="7"/>
       <c r="O11" s="8"/>
       <c r="P11" s="1"/>
@@ -2156,7 +2185,7 @@
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
     </row>
-    <row r="12" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="208.8" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>79</v>
       </c>
@@ -2181,13 +2210,21 @@
       <c r="H12" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I12" s="11"/>
-      <c r="J12" s="12"/>
+      <c r="I12" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="J12" s="12">
+        <v>1</v>
+      </c>
       <c r="K12" s="59" t="s">
         <v>230</v>
       </c>
-      <c r="L12" s="59"/>
-      <c r="M12" s="10"/>
+      <c r="L12" s="59" t="s">
+        <v>253</v>
+      </c>
+      <c r="M12" s="10" t="s">
+        <v>251</v>
+      </c>
       <c r="N12" s="10"/>
       <c r="O12" s="11"/>
       <c r="P12" s="1"/>
@@ -2202,7 +2239,7 @@
       <c r="Y12" s="1"/>
       <c r="Z12" s="1"/>
     </row>
-    <row r="13" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>86</v>
       </c>
@@ -2227,12 +2264,18 @@
       <c r="H13" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I13" s="8"/>
-      <c r="J13" s="9"/>
+      <c r="I13" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="J13" s="9">
+        <v>2</v>
+      </c>
       <c r="K13" s="58" t="s">
         <v>230</v>
       </c>
-      <c r="L13" s="58"/>
+      <c r="L13" s="58" t="s">
+        <v>252</v>
+      </c>
       <c r="M13" s="7"/>
       <c r="N13" s="7"/>
       <c r="O13" s="8"/>

</xml_diff>

<commit_message>
Finished up controls up to gap analysis
</commit_message>
<xml_diff>
--- a/compliance/Control_Matrix_Mapping.xlsx
+++ b/compliance/Control_Matrix_Mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kate\OneDrive\Documents\GRC_Risk_Assessment\C3-GRC\compliance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7090FAC3-5360-41A7-881D-61549FAE4AA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F5DE806-F38F-4CE2-B6AE-5B30ED1AF351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Control Matrix Mapping" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="254">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="287">
   <si>
     <t>CrochetCrochetCrochet (C3) — ISO 27001:2022 / NIST 800-53 Control Matrix</t>
   </si>
@@ -741,37 +741,13 @@
     <t>Y</t>
   </si>
   <si>
-    <t>Need SDLC offical documentation; Need additional security testing</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The control is operationally practiced, but not formally documented or communicated as a policy artifact. </t>
-  </si>
-  <si>
     <t>Microsoft Entra ID [C3-013] serves as the primary identity provider for C3, issuing and managing identities across all SSO-connected SaaS platforms including Microsoft 365, GitHub, 1Password, and Rippling. Each employee holds a unique Employee ID (EMP-001 through EMP-016) with a corresponding Entra ID identity. Iris Cohen (People &amp; Operations Coordinator) administers Rippling [C3-024], which manages the employee lifecycle including onboarding and offboarding workflows. Iris is noted as responsible for onboarding/offboarding access provisioning. No formal identity lifecycle management procedure was identified.</t>
-  </si>
-  <si>
-    <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C3-013]. Privileged accounts are required to use hardware security keys for any admin account activity. All credentials are stored and managed by 1Password [C3-020], with vault segmentation by department, preventing cross-functional exposure. No formal password policy is defined. No recovery procedures are defined.</t>
-  </si>
-  <si>
-    <t>Technical controls are in place via 1Password, however there are no formal policies or procedures in place for password policy, requirements, rotation scheduling, etc.</t>
-  </si>
-  <si>
-    <t>Role-based access control in implemented and operationally enforced through Microsoft Entra ID Conditional Access rules, [C3-013]. This governs authentication and device compliance requirements for all SaaS and cloud environment access. 1Password Teams  [C3-020] vaults are segmented by department, with credential access limited by function. Employee system access is provisioned per role. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts. No formal policy is identified or referenced.</t>
-  </si>
-  <si>
-    <t>Access provisioning follows the least-privilege model, by role-differentiated system access. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts.  1Password [C3-020] vault segmentation enforces access boundaries by department. No formal access rights review is documented, no procedures for access rights are documented.</t>
-  </si>
-  <si>
-    <t>Technical contros are in place via 1Password, however, no formal access rights review schedule, documented provisioning and deprovisioning procedures, or periodic recertification process have been identified beyond the noted quarterly review for privileged accounts.</t>
   </si>
   <si>
     <t xml:space="preserve">Partial </t>
   </si>
   <si>
     <t>There is no formal access control policy.</t>
-  </si>
-  <si>
-    <t>The control is operationally practiced, but not formally documented or communicated as a policy artifact.  The process appears to be operationally managed through Rippling and Entra ID but without a documented runbook defining steps, timelines, or verification requirements for provisioning and deprovisioning.</t>
   </si>
   <si>
     <t>Technical access restrictions are applied consitently across the infrastructure, despite the lack of documentation. The Production Customer DB [C3-002] is accessible via private VPC networking, with no public endpoint. The Admin Portal [C3-007] is restricted to VPN-only access [C3-0016] with MFA enforced and confirmed to be not publicly accessible. The Customer Uploads S3 bucket [C3-004] uses pre-signed URLs for time-limited access rather than direct bucket permissions. The Pattern Library S3 bucket [C3-003] has public read blocked at the bucket policy level. GitHub [C3-008] enforces private repositories only with branch protection enabled, requiring pull request review before any production deployment. CloudFront [C3-006] serves static assets with a WAF attached.</t>
@@ -789,37 +765,154 @@
     <t xml:space="preserve">Missing </t>
   </si>
   <si>
-    <t>No formal Information Security Policy document has been identified in the asset inventory, employee directory, or any referenced system notes. Security controls are operationally implemented across the environmen and ownership is assigned per control in this matrix. However, there is no evidence of a management-approved, published, and communicated information security policy that establishes C3's security intent, objectives, or responsibilities. The absence of this foundational document means all other controls lack a governing policy framework to reference, which represents a significant gap for any ISO 27001 audit.</t>
-  </si>
-  <si>
-    <t>Completely missing.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Regulatory awareness appears operationally embedded but not formally catalogued or reviewed on a defined schedule.</t>
-  </si>
-  <si>
     <t>PII is identified and flagged across the entire asset inventory using a dedicated 'Contains PII' column applied to all 42 assets. No formal Privacy Policy or PII handling procedure document has been identified. There is no documented process for responding to data subject access requests or right-to-erasure requests, which is a meaningful gap given C3's customer PII exposure and GDPR-adjacent obligations.</t>
   </si>
   <si>
-    <t>C3 operates in a regulatory environment touching multiple frameworks. PCI DSS obligations arise from subscription payment processing via Stripe [C3-012]; C3 mitigates direct PCI scope by tokenizing all payment card data through Stripe rather than storing raw card data. ISO 27001 compliance tags are applied to all 42 assets in the asset inventory. Customer PII and employee PII are present across multiple assets [C3-001, C3-002, C3-004, C3-015, C3-024], indicating GDPR and applicable U.S. privacy law obligations. Marcus Okafor is noted as responsible for finance and compliance-adjacent functions. No formal legal and regulatory register has been identified documenting all applicable obligations, their sources, review dates, or responsible owners</t>
+    <t>No security awareness training program has been identified. There is no reference to a training platform, completion tracking mechanism, training schedule, or role-based curriculum for any of C3's 16 employees. MFA and hardware key requirements are technically enforced at the tooling level, indicating some baseline security hygiene exists operationally. However, there is no evidence that staff have received formal instruction on phishing recognition, incident reporting, acceptable use, data handling, or any other security awareness topic.</t>
+  </si>
+  <si>
+    <t>Partially</t>
+  </si>
+  <si>
+    <t>No formal classification policy or labeling standard has been identified defining each tier's handling requirements or mandating consistent labeling on documents and files outside of the asset inventory context.</t>
+  </si>
+  <si>
+    <t>Jordan Ellis [DevOps &amp; Cloud Engineer, EMP-006] is identified as the Infrastructure-as-Code (IaC) owner, with all AWS infrastructure managed through IaC stored in the GitHub organization [C3-008]. GitHub Actions [C3-009) automates deployment pipelines and enforces consistent deployment processes, reducing manual configuration drift. Branch protection on GitHub requires pull request review before any infrastructure code change is applied, providing a change control mechanism. Microsoft Intune MDM [C3-010] manages endpoint configuration baselines for all 17 devices. Entra ID Conditional Access [C3-013] enforces compliant device requirements, acting as a soft configuration baseline gate.</t>
+  </si>
+  <si>
+    <t>No formal configuration baseline documentation has been identified for any asset class. There is no evidence of a configuration management policy, CIS Benchmark mappings, documented baseline standards, or drift detection reporting against which current configurations are measured.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The asset inventory tracks OS versions and patch status for all assets. Both production EC2 instances [C3-001, C3-007] are running Amazon Linux 2 version 2.0.20240131, noted as Current as of January 2025. Employee endpoints are all running macOS Sonoma 14.4, managed via Intune MDM. The Community Forum server [C3-018, Ubuntu 22.04 LTS] is explicitly flagged as 'Pending Patch' with a last review date of October 2024, representing a known and unresolved vulnerability as of the date of assessment, over three months overdue. </t>
+  </si>
+  <si>
+    <t>No dedicated vulnerability scanning tool (such as AWS Inspector, Tenable, or Qualys) is referenced in the asset inventory or system notes. There is no evidence of a formal vulnerability management policy, defined SLAs for patch remediation by severity, or a scheduled scanning cadence. The C3-018 overdue patch is a concrete, currently open vulnerability management failure.</t>
+  </si>
+  <si>
+    <t>No evidence of regular device compliance reporting or endpoint audit cadence has been found.</t>
+  </si>
+  <si>
+    <t>C3 relies on a significant number of third-party suppliers for core business functions, all catalogued in the asset inventory. Key suppliers include: AWS (cloud infrastructure), Microsoft (M365, Entra ID), GitHub (source control, CI/CD), Stripe (payment processing), Intercom (customer support), Rippling (HR and payroll), Mailchimp (email marketing), Canva (design), Figma (product design), and 1Password (secrets management). Stripe is noted as handling PCI scope on C3's behalf with webhook secrets rotated quarterly. GitHub is configured with SSO enforcement and secret scanning active.</t>
+  </si>
+  <si>
+    <t>No formal supplier security assessment process has been identified. There is no evidence of security questionnaires, data processing agreements (DPAs), contractual security clauses, or periodic supplier risk reviews for any third party. Supplier security is managed through platform configuration choices rather than a governed supplier risk management program.</t>
+  </si>
+  <si>
+    <t>AWS is C3's primary cloud provider, hosting the production web application [C3-001], customer database [C3-002], S3 storage buckets [C3-003, C3-004], load balancer [C3-005], CloudFront CDN [C3-006], admin portal [C3-007], VPN [C3-016], and community forum [C3-018]. Infrastructure is managed through IaC owned by Jordan Ellis and deployed via GitHub Actions [C3-009] using OIDC-based AWS credential passing rather than static keys. CloudWatch [C3-019] provides monitoring across AWS services. Multi-AZ is enabled for the production database. All cloud assets are tagged for ISO 27001 scope.</t>
+  </si>
+  <si>
+    <t>No formal cloud security policy has been identified covering approved cloud services, configuration standards, shared responsibility model acknowledgement, or cloud exit procedures. Cloud security decisions appear to be made at the engineering level without a governing policy framework.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No incident response plan, playbook, or incident management policy has been identified in the asset inventory, employee directory, or any system notes. CloudWatch [C3-019] generates alerts for failed logins and IAM changes, which could trigger an informal response, but no documented process exists defining what constitutes a security incident, how incidents are classified by severity, who is notified at each stage, what containment steps are taken, or how incidents are recorded and closed. No incident response roles or responsibilities have been assigned. No evidence of tabletop exercises or incident response testing has been found. </t>
+  </si>
+  <si>
+    <t>CloudWatch [C3-019] is configured to alert on failed logins and IAM changes, providing automated detection for a subset of security events at the AWS infrastructure layer. However, no formal channel or process exists for staff to report suspected security events. There is no reference to a security reporting email address, dedicated communication channel, ticketing queue, or escalation path for employees to use when they observe something suspicious. The Employee Directory and all system notes contain no reference to security event reporting procedures having been communicated to staff. Without a formal human reporting mechanism, events observed by employees, phishing attempts, accidental data disclosure, unauthorized access attempts, are likely to go unreported or handled inconsistently. Automated detection exists but human-initiated reporting capability is absent.</t>
+  </si>
+  <si>
+    <t>Several SDLC security practices are operationally in place. GitHub branch protection [C3-008] requires pull request review before any code merge, with Devon Nakamura's directory notes explicitly confirming 'no production deploy without PR review.' GitHub Actions [C3-009] automates testing and deployment pipelines. GitHub secret scanning is active to detect committed credentials. The CI/CD pipeline uses OIDC-based AWS credential passing rather than static secrets [C3-009]. No formal Secure Development Lifecycle policy or procedure document has been identified. There is no evidence of documented security requirements embedded in the development process, mandatory security testing gates (SAST, DAST, dependency scanning), threat modelling practices, or developer security training. SDLC security controls exist at the tooling level but are not governed by a formal policy or consistently applied framework.</t>
+  </si>
+  <si>
+    <t>Source code access is effectively controlled through the GitHub organization [C3-008]. All repositories are private with SSO enforced via Entra ID. Access is role-differentiated across the engineering team: Devon Nakamura and Jordan Ellis hold admin access; Sofia Reyes and Liam Huang hold write access; Camille Fontaine, Theo Mbeki, and Priya Sharma hold read or scoped read/write access appropriate to their roles. Branch protection is enabled, requiring pull request review before merges to protected branches. GitHub Actions [C3-009] handles automated deployment with AWS credentials passed via OIDC rather than stored as static repository secrets. Secret scanning is active across all repositories.</t>
+  </si>
+  <si>
+    <t>No formal log management policy has been identified defining required log sources, minimum retention periods per asset class, log integrity requirements, or procedures for log review and investigation. No centralized SIEM aggregating logs across SaaS, endpoints, and cloud has been identified.</t>
+  </si>
+  <si>
+    <t>Access provisioning follows the least-privilege model, by role-differentiated system access. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts. 1Password [C3-020] vault segmentation enforces access boundaries by department. No formal access rights review is documented, no procedures for access rights are documented.</t>
+  </si>
+  <si>
+    <t>Technical controls are in place via 1Password, however, no formal access rights review schedule, documented provisioning and deprovisioning procedures, or periodic recertification process have been identified beyond the noted quarterly review for privileged accounts.</t>
+  </si>
+  <si>
+    <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C3-013]. Privileged accounts are required to use hardware security keys for any admin account activity. All credentials are stored and managed by 1Password [C3-020], with vault segmentation by department, preventing cross-functional exposure.</t>
+  </si>
+  <si>
+    <t>No formal password policy is defined. No recovery procedures are defined. Technical controls are in place via 1Password.</t>
+  </si>
+  <si>
+    <t>No formal documentation was found.</t>
+  </si>
+  <si>
+    <t>C3 operates in a regulatory environment touching multiple frameworks. PCI DSS obligations arise from subscription payment processing via Stripe [C3-012]; C3 mitigates direct PCI scope by tokenizing all payment card data through Stripe rather than storing raw card data. ISO 27001 compliance tags are applied to all 42 assets in the asset inventory. Customer PII and employee PII are present across multiple assets [C3-001, C3-002, C3-004, C3-015, C3-024], indicating GDPR and applicable U.S. privacy law obligations. Marcus Okafor is noted as responsible for finance and compliance-adjacent functions.</t>
+  </si>
+  <si>
+    <t>Regulatory awareness appears operationally embedded but not formally catalogued or reviewed on a defined schedule. No formal legal and regulatory register has been identified documenting all applicable obligations, their sources, review dates, or responsible owners.</t>
+  </si>
+  <si>
+    <t>No formal Privacy Policy or PII handling procedure document has been identified. There is no documented process for responding to data subject access requests or right-to-erasure requests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No formal Information Security Policy document has been identified in the asset inventory, employee directory, or any referenced system notes. Security controls are operationally implemented across the environment and ownership is assigned per control in this matrix. However, there is no evidence of a management-approved, published, and communicated information security policy that establishes C3's security intent, objectives, or responsibilities. </t>
+  </si>
+  <si>
+    <t>C3 maintains a formal asset inventory covering 42 assets across five categories: cloud infrastructure [servers, databases, storage, networking), SaaS tools, identity and access management, payment processing, and employee endpoints. Each asset record includes Asset ID, Friendly Name, Asset Type, Asset Category, Business Owner, Technical Owner, Department, Custodian, Environment, Data Classification, Data Types Stored, PII and PCI flags, Sensitivity Score (1-5), ISO 27001 scope flag, Compliance Tags, Status, Date Added, and Last Updated. Asset IDs follow a consistent naming convention (C3-001 through C3-025 for infrastructure/SaaS; C3-EMP-001 through C3-EMP-016B for endpoints). One decommissioned asset (C3-017, Zoom, closed January 2025) is retained in the inventory with decommission date recorded. The inventory is actively maintained and comprehensive.</t>
+  </si>
+  <si>
+    <t>The formal asset inventory appears to be an accurate, living document, however, there is no formal procedure or policy outlining updating the inventory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Information classification is applied to all 42 assets in the asset inventory using a four-tier scheme: Restricted, Confidential, Internal, and Public. No assets are currently classified Public. Classification is recorded in a dedicated 'Data Classification' column for every asset. Restricted assets include the Production Database [C3-002], Admin Portal [C3-007], Stripe account [C3-012], Entra ID [C3-013], 1Password [C3-020], Rippling [C3-024], and QuickBooks [C3-025], all carrying sensitivity scores of 4 or 5. A supplementary 'Sensitivity Score (1-5)' column provides a numeric risk weighting alongside the classification label. Data types stored are documented per asset to support classification decisions. </t>
+  </si>
+  <si>
+    <t>All 17 endpoints are enrolled in Microsoft Intune MDM [C3-010], providing a baseline device compliance and configuration management layer. Endpoint Detection and Response (EDR) is explicitly confirmed on three high-risk devices: Devon Nakamura's MacBook Pro [C3-EMP-003, Full AWS Admin], Jordan Ellis's MacBook Pro [C3-EMP-006, AWS Admin / IaC owner], and Sofia Reyes's MacBook Pro [C3-EMP-004, Senior Software Engineer]. GitHub secret scanning [C3-008] is active to detect accidentally committed credentials. FileVault encryption is enabled on all macOS devices.</t>
+  </si>
+  <si>
+    <t>EDR coverage is not confirmed for the remaining 14 endpoints, including all MacBook Air devices assigned to Customer Success, Marketing, Operations, and Content staff. No anti-malware or EDR solution is referenced for the standard employee device fleet. There is no evidence of a centrally managed anti-malware policy, coverage reporting, or defined response procedure for malware detection events.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AWS CloudWatch [C3-019] provides centralized logging for all AWS services and application events, with log retention configured to one year. Alerting is configured for failed login attempts and IAM changes per C3-019 asset notes. The Corporate VPN [C3-016] retains connection logs for 90 days. GitHub Actions pipeline logs are reviewed quarterly per C3-009 notes. Community Forum moderation logs [C3-018] are retained for one year. Microsoft 365 and Teams [C3-010, C3-011] apply a one-year message retention policy with meeting recordings stored in OneDrive. Logging is implemented across the primary infrastructure stack. </t>
+  </si>
+  <si>
+    <t>AWS CloudWatch (C3-019) is the primary monitoring tool, configured with alerts for failed logins and IAM changes across the AWS environment. VPN connection logs (C3-016) are retained for 90 days and available for review. GitHub Actions pipeline logs are reviewed on a quarterly basis (C3-009). CloudFront (C3-006) has a WAF attached for traffic-level threat detection on the CDN layer. No Security Information and Event Management (SIEM) platform has been identified in the asset inventory.</t>
+  </si>
+  <si>
+    <t>There is no evidence of 24/7 monitoring coverage, a defined alert triage and response process, network traffic analysis beyond the WAF, or user behaviour analytics. Monitoring is reactive and infrastructure-focused. The absence of a SIEM means log correlation across SaaS platforms, endpoints, and cloud infrastructure is not currently occurring, and cross-source attack patterns would not be detected.</t>
+  </si>
+  <si>
+    <t>All 17 employee endpoints are enrolled in Microsoft Intune MDM via the M365 E3 tenant [C3-010], which enforces device compliance as a prerequisite for Entra ID Conditional Access. FileVault full-disk encryption is confirmed on all 16 MacBook devices. The iPad Pro [C3-EMP-016B] is enrolled under iPadOS 17.3. EDR is deployed on three high-risk MacBook Pros (CTO, DevOps Engineer, Senior Software Engineer). Hardware security keys are enforced on all admin-level devices. OS versions are consistent across the Mac fleet (macOS Sonoma 14.4). EDR coverage is confirmed for only 3 of 17 endpoints. No formal endpoint security policy or acceptable use policy has been identified. Screen lock enforcement is confirmed only on the CEO device (2 minutes); uniform enforcement across all 17 devices is not individually verified in the asset inventory.</t>
+  </si>
+  <si>
+    <t>Role-based access control in implemented and operationally enforced through Microsoft Entra ID Conditional Access rules, [C3-013]. This governs authentication and device compliance requirements for all SaaS and cloud environment access. 1Password Teams [C3-020] vaults are segmented by department, with credential access limited by function. Employee system access is provisioned per role. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No formal policy is identified or referenced. The control is operationally practiced, but not formally documented or communicated as a policy artifact. </t>
+  </si>
+  <si>
+    <t>The control is operationally practiced, but not formally documented or communicated as a policy artifact. The process appears to be operationally managed through Rippling and Entra ID but without a documented runbook defining steps, timelines, or verification requirements for provisioning and deprovisioning.</t>
+  </si>
+  <si>
+    <t>There is no security awareness training program. There is no evidence that staff have received formal instruction on phishing recognition, incident reporting, acceptable use, data handling, or any other security awareness topic.</t>
+  </si>
+  <si>
+    <t>Iris Cohen [People &amp; Operations Coordinator, EMP-015] is identified as the owner of onboarding and offboarding access provisioning, supported by Rippling [C3-024] as the HRIS platform. Entra ID [C3-013] is the central identity provider, meaning account deprovisioning through Entra ID cascades to all SSO-connected platforms. The Employee Directory notes that access reviews are conducted at each offboarding event. Devon Nakamura is noted for quarterly access reviews on privileged accounts.</t>
+  </si>
+  <si>
+    <t>The control is operationally practiced but undocumented, creating risk of inconsistent execution. No formal offboarding procedure document has been identified specifying timelines for access revocation, defining which systems require manual deprovisioning beyond SSO, establishing verification steps, or addressing equipment return and data handling for departing employees.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">No incident response plan, playbook, or incident management policy has been identified in the asset inventory, employee directory, or any system notes. No documented process exists defining what constitutes a security incident, how incidents are classified by severity, who is notified at each stage, what containment steps are taken, or how incidents are recorded and closed. No incident response roles or responsibilities have been assigned. No evidence of tabletop exercises or incident response testing has been found. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">No formal channel or process exists for staff to report suspected security events. There is no reference to a security reporting email address, dedicated communication channel, ticketing queue, or escalation path for employees to use when they observe something suspicious. The Employee Directory and all system notes contain no reference to security event reporting procedures having been communicated to staff. </t>
+  </si>
+  <si>
+    <t>There is no evidence of documented security requirements embedded in the development process, mandatory security testing gates (SAST, DAST, dependency scanning), threat modelling practices, or developer security training. SDLC security controls exist at the tooling level but are not governed by a formal policy or consistently applied framework.</t>
+  </si>
+  <si>
+    <t>Secure code access is effectively controlled through GitHub, however, there is no formal procedure or policy documentation.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
     </font>
     <font>
       <sz val="10"/>
@@ -966,6 +1059,20 @@
       <sz val="8"/>
       <name val="Arial"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="29">
@@ -1202,190 +1309,193 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="22" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="22" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="24" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="16" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="17" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="26" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="15" fillId="23" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="24" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="24" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="17" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="19" fillId="18" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="8" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="23" fillId="9" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="25" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="11" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1608,39 +1718,39 @@
   <dimension ref="A1:Z995"/>
   <sheetFormatPr defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="23.77734375" style="73" customWidth="1"/>
-    <col min="2" max="2" width="13.6640625" style="73" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" style="73" customWidth="1"/>
-    <col min="4" max="4" width="14" style="73" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" style="73" customWidth="1"/>
-    <col min="6" max="6" width="12.6640625" style="73"/>
-    <col min="7" max="7" width="45.33203125" style="73" customWidth="1"/>
-    <col min="8" max="8" width="10.77734375" style="73" customWidth="1"/>
-    <col min="9" max="11" width="12.6640625" style="73"/>
-    <col min="12" max="12" width="33.88671875" style="73" customWidth="1"/>
-    <col min="13" max="13" width="28.109375" style="73" customWidth="1"/>
-    <col min="14" max="14" width="24.33203125" style="73" customWidth="1"/>
-    <col min="15" max="16384" width="12.6640625" style="73"/>
+    <col min="1" max="1" width="23.77734375" style="66" customWidth="1"/>
+    <col min="2" max="2" width="13.6640625" style="66" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" style="66" customWidth="1"/>
+    <col min="4" max="4" width="14" style="66" hidden="1" customWidth="1"/>
+    <col min="5" max="5" width="16.33203125" style="66" customWidth="1"/>
+    <col min="6" max="6" width="12.6640625" style="66"/>
+    <col min="7" max="7" width="45.33203125" style="66" customWidth="1"/>
+    <col min="8" max="8" width="10.77734375" style="66" customWidth="1"/>
+    <col min="9" max="11" width="12.6640625" style="66"/>
+    <col min="12" max="12" width="55.109375" style="66" customWidth="1"/>
+    <col min="13" max="13" width="40.21875" style="66" customWidth="1"/>
+    <col min="14" max="14" width="24.33203125" style="66" customWidth="1"/>
+    <col min="15" max="16384" width="12.6640625" style="66"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="66" t="s">
+    <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="71"/>
-      <c r="C1" s="71"/>
-      <c r="D1" s="71"/>
-      <c r="E1" s="71"/>
-      <c r="F1" s="71"/>
-      <c r="G1" s="71"/>
-      <c r="H1" s="71"/>
-      <c r="I1" s="71"/>
-      <c r="J1" s="71"/>
-      <c r="K1" s="71"/>
-      <c r="L1" s="71"/>
-      <c r="M1" s="71"/>
-      <c r="N1" s="71"/>
-      <c r="O1" s="72"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67"/>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="68"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -1653,30 +1763,30 @@
       <c r="Y1" s="1"/>
       <c r="Z1" s="1"/>
     </row>
-    <row r="2" spans="1:26" ht="21" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="67" t="s">
+    <row r="2" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="69" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="72"/>
-      <c r="F2" s="68" t="s">
+      <c r="B2" s="67"/>
+      <c r="C2" s="67"/>
+      <c r="D2" s="67"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="70" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="72"/>
-      <c r="H2" s="69" t="s">
+      <c r="G2" s="68"/>
+      <c r="H2" s="71" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="71"/>
-      <c r="J2" s="71"/>
-      <c r="K2" s="71"/>
-      <c r="L2" s="72"/>
-      <c r="M2" s="70" t="s">
+      <c r="I2" s="67"/>
+      <c r="J2" s="67"/>
+      <c r="K2" s="67"/>
+      <c r="L2" s="68"/>
+      <c r="M2" s="72" t="s">
         <v>4</v>
       </c>
-      <c r="N2" s="71"/>
-      <c r="O2" s="72"/>
+      <c r="N2" s="67"/>
+      <c r="O2" s="68"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -1805,7 +1915,7 @@
       <c r="Y4" s="1"/>
       <c r="Z4" s="1"/>
     </row>
-    <row r="5" spans="1:26" ht="148.19999999999999" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" ht="79.8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>35</v>
       </c>
@@ -1839,11 +1949,11 @@
       <c r="K5" s="58" t="s">
         <v>227</v>
       </c>
-      <c r="L5" s="58" t="s">
-        <v>238</v>
-      </c>
-      <c r="M5" s="7" t="s">
-        <v>234</v>
+      <c r="L5" s="62" t="s">
+        <v>277</v>
+      </c>
+      <c r="M5" s="61" t="s">
+        <v>278</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="8"/>
@@ -1859,7 +1969,7 @@
       <c r="Y5" s="1"/>
       <c r="Z5" s="1"/>
     </row>
-    <row r="6" spans="1:26" ht="182.4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>42</v>
       </c>
@@ -1885,7 +1995,7 @@
         <v>232</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="J6" s="12">
         <v>2</v>
@@ -1893,11 +2003,11 @@
       <c r="K6" s="59" t="s">
         <v>228</v>
       </c>
-      <c r="L6" s="59" t="s">
-        <v>235</v>
-      </c>
-      <c r="M6" s="10" t="s">
-        <v>243</v>
+      <c r="L6" s="63" t="s">
+        <v>233</v>
+      </c>
+      <c r="M6" s="64" t="s">
+        <v>279</v>
       </c>
       <c r="N6" s="10"/>
       <c r="O6" s="11"/>
@@ -1913,7 +2023,7 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" ht="114" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="57" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>48</v>
       </c>
@@ -1939,7 +2049,7 @@
         <v>232</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>241</v>
+        <v>234</v>
       </c>
       <c r="J7" s="9">
         <v>2</v>
@@ -1947,11 +2057,11 @@
       <c r="K7" s="58" t="s">
         <v>227</v>
       </c>
-      <c r="L7" s="58" t="s">
-        <v>236</v>
-      </c>
-      <c r="M7" s="7" t="s">
-        <v>237</v>
+      <c r="L7" s="62" t="s">
+        <v>261</v>
+      </c>
+      <c r="M7" s="61" t="s">
+        <v>262</v>
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="8"/>
@@ -1967,7 +2077,7 @@
       <c r="Y7" s="1"/>
       <c r="Z7" s="1"/>
     </row>
-    <row r="8" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" ht="84" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>54</v>
       </c>
@@ -2001,11 +2111,11 @@
       <c r="K8" s="59" t="s">
         <v>227</v>
       </c>
-      <c r="L8" s="59" t="s">
-        <v>239</v>
-      </c>
-      <c r="M8" s="10" t="s">
-        <v>240</v>
+      <c r="L8" s="63" t="s">
+        <v>259</v>
+      </c>
+      <c r="M8" s="64" t="s">
+        <v>260</v>
       </c>
       <c r="N8" s="10"/>
       <c r="O8" s="11"/>
@@ -2021,7 +2131,7 @@
       <c r="Y8" s="1"/>
       <c r="Z8" s="1"/>
     </row>
-    <row r="9" spans="1:26" ht="216.6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" ht="136.80000000000001" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>60</v>
       </c>
@@ -2055,14 +2165,14 @@
       <c r="K9" s="58" t="s">
         <v>227</v>
       </c>
-      <c r="L9" s="58" t="s">
-        <v>244</v>
+      <c r="L9" s="62" t="s">
+        <v>236</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="N9" s="7" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="O9" s="8"/>
       <c r="P9" s="1"/>
@@ -2077,7 +2187,7 @@
       <c r="Y9" s="1"/>
       <c r="Z9" s="1"/>
     </row>
-    <row r="10" spans="1:26" ht="125.4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" ht="79.8" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
         <v>66</v>
       </c>
@@ -2112,10 +2222,10 @@
         <v>227</v>
       </c>
       <c r="L10" s="63" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="M10" s="64" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="N10" s="10"/>
       <c r="O10" s="11"/>
@@ -2131,7 +2241,7 @@
       <c r="Y10" s="1"/>
       <c r="Z10" s="1"/>
     </row>
-    <row r="11" spans="1:26" ht="182.4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" ht="79.8" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>72</v>
       </c>
@@ -2157,7 +2267,7 @@
         <v>232</v>
       </c>
       <c r="I11" s="60" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="J11" s="9">
         <v>1</v>
@@ -2165,11 +2275,11 @@
       <c r="K11" s="58" t="s">
         <v>229</v>
       </c>
-      <c r="L11" s="58" t="s">
-        <v>249</v>
-      </c>
-      <c r="M11" s="7" t="s">
-        <v>250</v>
+      <c r="L11" s="62" t="s">
+        <v>267</v>
+      </c>
+      <c r="M11" s="61" t="s">
+        <v>263</v>
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="8"/>
@@ -2185,7 +2295,7 @@
       <c r="Y11" s="1"/>
       <c r="Z11" s="1"/>
     </row>
-    <row r="12" spans="1:26" ht="208.8" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
         <v>79</v>
       </c>
@@ -2211,7 +2321,7 @@
         <v>232</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="J12" s="12">
         <v>1</v>
@@ -2219,11 +2329,11 @@
       <c r="K12" s="59" t="s">
         <v>230</v>
       </c>
-      <c r="L12" s="59" t="s">
-        <v>253</v>
-      </c>
-      <c r="M12" s="10" t="s">
-        <v>251</v>
+      <c r="L12" s="63" t="s">
+        <v>264</v>
+      </c>
+      <c r="M12" s="64" t="s">
+        <v>265</v>
       </c>
       <c r="N12" s="10"/>
       <c r="O12" s="11"/>
@@ -2239,7 +2349,7 @@
       <c r="Y12" s="1"/>
       <c r="Z12" s="1"/>
     </row>
-    <row r="13" spans="1:26" ht="114" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:26" ht="68.400000000000006" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
         <v>86</v>
       </c>
@@ -2273,10 +2383,12 @@
       <c r="K13" s="58" t="s">
         <v>230</v>
       </c>
-      <c r="L13" s="58" t="s">
-        <v>252</v>
-      </c>
-      <c r="M13" s="7"/>
+      <c r="L13" s="62" t="s">
+        <v>241</v>
+      </c>
+      <c r="M13" s="61" t="s">
+        <v>266</v>
+      </c>
       <c r="N13" s="7"/>
       <c r="O13" s="8"/>
       <c r="P13" s="1"/>
@@ -2291,7 +2403,7 @@
       <c r="Y13" s="1"/>
       <c r="Z13" s="1"/>
     </row>
-    <row r="14" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:26" ht="148.19999999999999" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
         <v>93</v>
       </c>
@@ -2316,13 +2428,21 @@
       <c r="H14" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I14" s="11"/>
-      <c r="J14" s="12"/>
+      <c r="I14" s="11" t="s">
+        <v>196</v>
+      </c>
+      <c r="J14" s="12">
+        <v>4</v>
+      </c>
       <c r="K14" s="59" t="s">
         <v>231</v>
       </c>
-      <c r="L14" s="59"/>
-      <c r="M14" s="10"/>
+      <c r="L14" s="63" t="s">
+        <v>268</v>
+      </c>
+      <c r="M14" s="64" t="s">
+        <v>269</v>
+      </c>
       <c r="N14" s="10"/>
       <c r="O14" s="11"/>
       <c r="P14" s="1"/>
@@ -2337,7 +2457,7 @@
       <c r="Y14" s="1"/>
       <c r="Z14" s="1"/>
     </row>
-    <row r="15" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
         <v>100</v>
       </c>
@@ -2362,13 +2482,21 @@
       <c r="H15" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I15" s="8"/>
-      <c r="J15" s="9"/>
+      <c r="I15" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="J15" s="9">
+        <v>2</v>
+      </c>
       <c r="K15" s="58" t="s">
         <v>230</v>
       </c>
-      <c r="L15" s="58"/>
-      <c r="M15" s="7"/>
+      <c r="L15" s="62" t="s">
+        <v>270</v>
+      </c>
+      <c r="M15" s="7" t="s">
+        <v>244</v>
+      </c>
       <c r="N15" s="7"/>
       <c r="O15" s="8"/>
       <c r="P15" s="1"/>
@@ -2383,7 +2511,7 @@
       <c r="Y15" s="1"/>
       <c r="Z15" s="1"/>
     </row>
-    <row r="16" spans="1:26" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:26" ht="91.2" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
         <v>106</v>
       </c>
@@ -2408,13 +2536,21 @@
       <c r="H16" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I16" s="11"/>
-      <c r="J16" s="12"/>
+      <c r="I16" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="J16" s="12">
+        <v>1</v>
+      </c>
       <c r="K16" s="59" t="s">
         <v>228</v>
       </c>
-      <c r="L16" s="59"/>
-      <c r="M16" s="10"/>
+      <c r="L16" s="63" t="s">
+        <v>242</v>
+      </c>
+      <c r="M16" s="64" t="s">
+        <v>280</v>
+      </c>
       <c r="N16" s="10"/>
       <c r="O16" s="11"/>
       <c r="P16" s="1"/>
@@ -2429,7 +2565,7 @@
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
     </row>
-    <row r="17" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>113</v>
       </c>
@@ -2454,13 +2590,21 @@
       <c r="H17" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I17" s="8"/>
-      <c r="J17" s="9"/>
+      <c r="I17" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="J17" s="9">
+        <v>2</v>
+      </c>
       <c r="K17" s="58" t="s">
         <v>228</v>
       </c>
-      <c r="L17" s="58"/>
-      <c r="M17" s="7"/>
+      <c r="L17" s="62" t="s">
+        <v>281</v>
+      </c>
+      <c r="M17" s="61" t="s">
+        <v>282</v>
+      </c>
       <c r="N17" s="7"/>
       <c r="O17" s="8"/>
       <c r="P17" s="1"/>
@@ -2475,7 +2619,7 @@
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
     </row>
-    <row r="18" spans="1:26" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>119</v>
       </c>
@@ -2500,13 +2644,21 @@
       <c r="H18" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I18" s="8"/>
-      <c r="J18" s="9"/>
+      <c r="I18" s="8" t="s">
+        <v>198</v>
+      </c>
+      <c r="J18" s="9">
+        <v>1</v>
+      </c>
       <c r="K18" s="58" t="s">
         <v>231</v>
       </c>
-      <c r="L18" s="58"/>
-      <c r="M18" s="7"/>
+      <c r="L18" s="62" t="s">
+        <v>271</v>
+      </c>
+      <c r="M18" s="61" t="s">
+        <v>272</v>
+      </c>
       <c r="N18" s="7"/>
       <c r="O18" s="8"/>
       <c r="P18" s="1"/>
@@ -2521,7 +2673,7 @@
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
     </row>
-    <row r="19" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
         <v>120</v>
       </c>
@@ -2546,13 +2698,21 @@
       <c r="H19" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I19" s="11"/>
-      <c r="J19" s="12"/>
+      <c r="I19" s="11" t="s">
+        <v>200</v>
+      </c>
+      <c r="J19" s="12">
+        <v>1</v>
+      </c>
       <c r="K19" s="59" t="s">
         <v>227</v>
       </c>
-      <c r="L19" s="59"/>
-      <c r="M19" s="10"/>
+      <c r="L19" s="63" t="s">
+        <v>247</v>
+      </c>
+      <c r="M19" s="64" t="s">
+        <v>248</v>
+      </c>
       <c r="N19" s="10"/>
       <c r="O19" s="11"/>
       <c r="P19" s="1"/>
@@ -2567,7 +2727,7 @@
       <c r="Y19" s="1"/>
       <c r="Z19" s="1"/>
     </row>
-    <row r="20" spans="1:26" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>127</v>
       </c>
@@ -2592,13 +2752,21 @@
       <c r="H20" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I20" s="8"/>
-      <c r="J20" s="9"/>
+      <c r="I20" s="8" t="s">
+        <v>200</v>
+      </c>
+      <c r="J20" s="9">
+        <v>1</v>
+      </c>
       <c r="K20" s="58" t="s">
         <v>231</v>
       </c>
-      <c r="L20" s="58"/>
-      <c r="M20" s="7"/>
+      <c r="L20" s="63" t="s">
+        <v>245</v>
+      </c>
+      <c r="M20" s="7" t="s">
+        <v>246</v>
+      </c>
       <c r="N20" s="7"/>
       <c r="O20" s="8"/>
       <c r="P20" s="1"/>
@@ -2613,7 +2781,7 @@
       <c r="Y20" s="1"/>
       <c r="Z20" s="1"/>
     </row>
-    <row r="21" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>133</v>
       </c>
@@ -2638,13 +2806,21 @@
       <c r="H21" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I21" s="11"/>
-      <c r="J21" s="12"/>
+      <c r="I21" s="65" t="s">
+        <v>198</v>
+      </c>
+      <c r="J21" s="12">
+        <v>2</v>
+      </c>
       <c r="K21" s="59" t="s">
         <v>231</v>
       </c>
-      <c r="L21" s="59"/>
-      <c r="M21" s="10"/>
+      <c r="L21" s="73" t="s">
+        <v>273</v>
+      </c>
+      <c r="M21" s="64" t="s">
+        <v>258</v>
+      </c>
       <c r="N21" s="10"/>
       <c r="O21" s="11"/>
       <c r="P21" s="1"/>
@@ -2659,7 +2835,7 @@
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
     </row>
-    <row r="22" spans="1:26" ht="22.8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" ht="125.4" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>139</v>
       </c>
@@ -2689,8 +2865,12 @@
       <c r="K22" s="58" t="s">
         <v>231</v>
       </c>
-      <c r="L22" s="58"/>
-      <c r="M22" s="7"/>
+      <c r="L22" s="62" t="s">
+        <v>274</v>
+      </c>
+      <c r="M22" s="61" t="s">
+        <v>275</v>
+      </c>
       <c r="N22" s="7"/>
       <c r="O22" s="8"/>
       <c r="P22" s="1"/>
@@ -2705,7 +2885,7 @@
       <c r="Y22" s="1"/>
       <c r="Z22" s="1"/>
     </row>
-    <row r="23" spans="1:26" ht="24" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:26" ht="136.80000000000001" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>145</v>
       </c>
@@ -2730,13 +2910,21 @@
       <c r="H23" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I23" s="8"/>
-      <c r="J23" s="9"/>
+      <c r="I23" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="J23" s="9">
+        <v>1</v>
+      </c>
       <c r="K23" s="58" t="s">
         <v>231</v>
       </c>
-      <c r="L23" s="58"/>
-      <c r="M23" s="7"/>
+      <c r="L23" s="62" t="s">
+        <v>276</v>
+      </c>
+      <c r="M23" s="61" t="s">
+        <v>249</v>
+      </c>
       <c r="N23" s="7"/>
       <c r="O23" s="8"/>
       <c r="P23" s="1"/>
@@ -2751,7 +2939,7 @@
       <c r="Y23" s="1"/>
       <c r="Z23" s="1"/>
     </row>
-    <row r="24" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>151</v>
       </c>
@@ -2776,13 +2964,21 @@
       <c r="H24" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I24" s="11"/>
-      <c r="J24" s="12"/>
+      <c r="I24" s="65" t="s">
+        <v>200</v>
+      </c>
+      <c r="J24" s="12">
+        <v>1</v>
+      </c>
       <c r="K24" s="59" t="s">
         <v>230</v>
       </c>
-      <c r="L24" s="59"/>
-      <c r="M24" s="10"/>
+      <c r="L24" s="63" t="s">
+        <v>250</v>
+      </c>
+      <c r="M24" s="64" t="s">
+        <v>251</v>
+      </c>
       <c r="N24" s="10"/>
       <c r="O24" s="11"/>
       <c r="P24" s="1"/>
@@ -2797,7 +2993,7 @@
       <c r="Y24" s="1"/>
       <c r="Z24" s="1"/>
     </row>
-    <row r="25" spans="1:26" ht="24" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>152</v>
       </c>
@@ -2822,13 +3018,21 @@
       <c r="H25" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I25" s="8"/>
-      <c r="J25" s="9"/>
+      <c r="I25" s="60" t="s">
+        <v>200</v>
+      </c>
+      <c r="J25" s="9">
+        <v>1</v>
+      </c>
       <c r="K25" s="58" t="s">
         <v>231</v>
       </c>
-      <c r="L25" s="58"/>
-      <c r="M25" s="7"/>
+      <c r="L25" s="62" t="s">
+        <v>252</v>
+      </c>
+      <c r="M25" s="61" t="s">
+        <v>253</v>
+      </c>
       <c r="N25" s="7"/>
       <c r="O25" s="8"/>
       <c r="P25" s="1"/>
@@ -2843,7 +3047,7 @@
       <c r="Y25" s="1"/>
       <c r="Z25" s="1"/>
     </row>
-    <row r="26" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" ht="125.4" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>159</v>
       </c>
@@ -2868,13 +3072,21 @@
       <c r="H26" s="10" t="s">
         <v>232</v>
       </c>
-      <c r="I26" s="11"/>
-      <c r="J26" s="12"/>
+      <c r="I26" s="65" t="s">
+        <v>200</v>
+      </c>
+      <c r="J26" s="12">
+        <v>1</v>
+      </c>
       <c r="K26" s="59" t="s">
         <v>227</v>
       </c>
-      <c r="L26" s="59"/>
-      <c r="M26" s="10"/>
+      <c r="L26" s="63" t="s">
+        <v>254</v>
+      </c>
+      <c r="M26" s="64" t="s">
+        <v>283</v>
+      </c>
       <c r="N26" s="10"/>
       <c r="O26" s="11"/>
       <c r="P26" s="1"/>
@@ -2889,7 +3101,7 @@
       <c r="Y26" s="1"/>
       <c r="Z26" s="1"/>
     </row>
-    <row r="27" spans="1:26" ht="24" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:26" ht="148.19999999999999" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>166</v>
       </c>
@@ -2914,13 +3126,21 @@
       <c r="H27" s="7" t="s">
         <v>232</v>
       </c>
-      <c r="I27" s="8"/>
-      <c r="J27" s="9"/>
+      <c r="I27" s="60" t="s">
+        <v>198</v>
+      </c>
+      <c r="J27" s="9">
+        <v>2</v>
+      </c>
       <c r="K27" s="58" t="s">
         <v>227</v>
       </c>
-      <c r="L27" s="58"/>
-      <c r="M27" s="7"/>
+      <c r="L27" s="62" t="s">
+        <v>255</v>
+      </c>
+      <c r="M27" s="61" t="s">
+        <v>284</v>
+      </c>
       <c r="N27" s="7"/>
       <c r="O27" s="8"/>
       <c r="P27" s="1"/>
@@ -2935,7 +3155,7 @@
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
     </row>
-    <row r="28" spans="1:26" ht="34.200000000000003" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" ht="148.19999999999999" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>170</v>
       </c>
@@ -2963,13 +3183,17 @@
       <c r="I28" s="60" t="s">
         <v>198</v>
       </c>
-      <c r="J28" s="9"/>
+      <c r="J28" s="9">
+        <v>2</v>
+      </c>
       <c r="K28" s="58" t="s">
         <v>227</v>
       </c>
-      <c r="L28" s="62"/>
+      <c r="L28" s="62" t="s">
+        <v>256</v>
+      </c>
       <c r="M28" s="61" t="s">
-        <v>233</v>
+        <v>285</v>
       </c>
       <c r="N28" s="7"/>
       <c r="O28" s="8"/>
@@ -2985,7 +3209,7 @@
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
     </row>
-    <row r="29" spans="1:26" ht="24" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>177</v>
       </c>
@@ -3013,12 +3237,18 @@
       <c r="I29" s="11" t="s">
         <v>196</v>
       </c>
-      <c r="J29" s="12"/>
+      <c r="J29" s="12">
+        <v>4</v>
+      </c>
       <c r="K29" s="59" t="s">
         <v>227</v>
       </c>
-      <c r="L29" s="59"/>
-      <c r="M29" s="10"/>
+      <c r="L29" s="63" t="s">
+        <v>257</v>
+      </c>
+      <c r="M29" s="64" t="s">
+        <v>286</v>
+      </c>
       <c r="N29" s="10"/>
       <c r="O29" s="11"/>
       <c r="P29" s="1"/>
@@ -30059,7 +30289,7 @@
     <mergeCell ref="H2:L2"/>
     <mergeCell ref="M2:O2"/>
   </mergeCells>
-  <phoneticPr fontId="27" type="noConversion"/>
+  <phoneticPr fontId="26" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Typos, Corrections, adding Depth/Risk Consequence. Still on Gap descriptions
</commit_message>
<xml_diff>
--- a/compliance/Control_Matrix_Mapping.xlsx
+++ b/compliance/Control_Matrix_Mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kate\OneDrive\Documents\GRC_Risk_Assessment\C3-GRC\compliance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9F5DE806-F38F-4CE2-B6AE-5B30ED1AF351}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EDA40CE-F714-4E1E-BF25-9B052CD94C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Control Matrix Mapping" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="368" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="286">
   <si>
     <t>CrochetCrochetCrochet (C3) — ISO 27001:2022 / NIST 800-53 Control Matrix</t>
   </si>
@@ -136,9 +136,6 @@
   </si>
   <si>
     <t>What evidence did you find? What is currently in place?</t>
-  </si>
-  <si>
-    <t>What is the specific gap you identified?</t>
   </si>
   <si>
     <t>What concrete steps would close the gap?</t>
@@ -750,9 +747,6 @@
     <t>There is no formal access control policy.</t>
   </si>
   <si>
-    <t>Technical access restrictions are applied consitently across the infrastructure, despite the lack of documentation. The Production Customer DB [C3-002] is accessible via private VPC networking, with no public endpoint. The Admin Portal [C3-007] is restricted to VPN-only access [C3-0016] with MFA enforced and confirmed to be not publicly accessible. The Customer Uploads S3 bucket [C3-004] uses pre-signed URLs for time-limited access rather than direct bucket permissions. The Pattern Library S3 bucket [C3-003] has public read blocked at the bucket policy level. GitHub [C3-008] enforces private repositories only with branch protection enabled, requiring pull request review before any production deployment. CloudFront [C3-006] serves static assets with a WAF attached.</t>
-  </si>
-  <si>
     <t>Develop a formal access control policy.</t>
   </si>
   <si>
@@ -765,13 +759,7 @@
     <t xml:space="preserve">Missing </t>
   </si>
   <si>
-    <t>PII is identified and flagged across the entire asset inventory using a dedicated 'Contains PII' column applied to all 42 assets. No formal Privacy Policy or PII handling procedure document has been identified. There is no documented process for responding to data subject access requests or right-to-erasure requests, which is a meaningful gap given C3's customer PII exposure and GDPR-adjacent obligations.</t>
-  </si>
-  <si>
     <t>No security awareness training program has been identified. There is no reference to a training platform, completion tracking mechanism, training schedule, or role-based curriculum for any of C3's 16 employees. MFA and hardware key requirements are technically enforced at the tooling level, indicating some baseline security hygiene exists operationally. However, there is no evidence that staff have received formal instruction on phishing recognition, incident reporting, acceptable use, data handling, or any other security awareness topic.</t>
-  </si>
-  <si>
-    <t>Partially</t>
   </si>
   <si>
     <t>No formal classification policy or labeling standard has been identified defining each tier's handling requirements or mandating consistent labeling on documents and files outside of the asset inventory context.</t>
@@ -819,19 +807,7 @@
     <t>No formal log management policy has been identified defining required log sources, minimum retention periods per asset class, log integrity requirements, or procedures for log review and investigation. No centralized SIEM aggregating logs across SaaS, endpoints, and cloud has been identified.</t>
   </si>
   <si>
-    <t>Access provisioning follows the least-privilege model, by role-differentiated system access. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts. 1Password [C3-020] vault segmentation enforces access boundaries by department. No formal access rights review is documented, no procedures for access rights are documented.</t>
-  </si>
-  <si>
     <t>Technical controls are in place via 1Password, however, no formal access rights review schedule, documented provisioning and deprovisioning procedures, or periodic recertification process have been identified beyond the noted quarterly review for privileged accounts.</t>
-  </si>
-  <si>
-    <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C3-013]. Privileged accounts are required to use hardware security keys for any admin account activity. All credentials are stored and managed by 1Password [C3-020], with vault segmentation by department, preventing cross-functional exposure.</t>
-  </si>
-  <si>
-    <t>No formal password policy is defined. No recovery procedures are defined. Technical controls are in place via 1Password.</t>
-  </si>
-  <si>
-    <t>No formal documentation was found.</t>
   </si>
   <si>
     <t>C3 operates in a regulatory environment touching multiple frameworks. PCI DSS obligations arise from subscription payment processing via Stripe [C3-012]; C3 mitigates direct PCI scope by tokenizing all payment card data through Stripe rather than storing raw card data. ISO 27001 compliance tags are applied to all 42 assets in the asset inventory. Customer PII and employee PII are present across multiple assets [C3-001, C3-002, C3-004, C3-015, C3-024], indicating GDPR and applicable U.S. privacy law obligations. Marcus Okafor is noted as responsible for finance and compliance-adjacent functions.</t>
@@ -858,9 +834,6 @@
     <t>All 17 endpoints are enrolled in Microsoft Intune MDM [C3-010], providing a baseline device compliance and configuration management layer. Endpoint Detection and Response (EDR) is explicitly confirmed on three high-risk devices: Devon Nakamura's MacBook Pro [C3-EMP-003, Full AWS Admin], Jordan Ellis's MacBook Pro [C3-EMP-006, AWS Admin / IaC owner], and Sofia Reyes's MacBook Pro [C3-EMP-004, Senior Software Engineer]. GitHub secret scanning [C3-008] is active to detect accidentally committed credentials. FileVault encryption is enabled on all macOS devices.</t>
   </si>
   <si>
-    <t>EDR coverage is not confirmed for the remaining 14 endpoints, including all MacBook Air devices assigned to Customer Success, Marketing, Operations, and Content staff. No anti-malware or EDR solution is referenced for the standard employee device fleet. There is no evidence of a centrally managed anti-malware policy, coverage reporting, or defined response procedure for malware detection events.</t>
-  </si>
-  <si>
     <t xml:space="preserve">AWS CloudWatch [C3-019] provides centralized logging for all AWS services and application events, with log retention configured to one year. Alerting is configured for failed login attempts and IAM changes per C3-019 asset notes. The Corporate VPN [C3-016] retains connection logs for 90 days. GitHub Actions pipeline logs are reviewed quarterly per C3-009 notes. Community Forum moderation logs [C3-018] are retained for one year. Microsoft 365 and Teams [C3-010, C3-011] apply a one-year message retention policy with meeting recordings stored in OneDrive. Logging is implemented across the primary infrastructure stack. </t>
   </si>
   <si>
@@ -871,9 +844,6 @@
   </si>
   <si>
     <t>All 17 employee endpoints are enrolled in Microsoft Intune MDM via the M365 E3 tenant [C3-010], which enforces device compliance as a prerequisite for Entra ID Conditional Access. FileVault full-disk encryption is confirmed on all 16 MacBook devices. The iPad Pro [C3-EMP-016B] is enrolled under iPadOS 17.3. EDR is deployed on three high-risk MacBook Pros (CTO, DevOps Engineer, Senior Software Engineer). Hardware security keys are enforced on all admin-level devices. OS versions are consistent across the Mac fleet (macOS Sonoma 14.4). EDR coverage is confirmed for only 3 of 17 endpoints. No formal endpoint security policy or acceptable use policy has been identified. Screen lock enforcement is confirmed only on the CEO device (2 minutes); uniform enforcement across all 17 devices is not individually verified in the asset inventory.</t>
-  </si>
-  <si>
-    <t>Role-based access control in implemented and operationally enforced through Microsoft Entra ID Conditional Access rules, [C3-013]. This governs authentication and device compliance requirements for all SaaS and cloud environment access. 1Password Teams [C3-020] vaults are segmented by department, with credential access limited by function. Employee system access is provisioned per role. Devon Nakamura is noted as responsible for quartly access reviews on privleged accounts.</t>
   </si>
   <si>
     <t xml:space="preserve">No formal policy is identified or referenced. The control is operationally practiced, but not formally documented or communicated as a policy artifact. </t>
@@ -901,6 +871,33 @@
   </si>
   <si>
     <t>Secure code access is effectively controlled through GitHub, however, there is no formal procedure or policy documentation.</t>
+  </si>
+  <si>
+    <t>Technical access restrictions are applied consistently across the infrastructure, despite the lack of documentation. The Production Customer DB [C3-002] is accessible via private VPC networking, with no public endpoint. The Admin Portal [C3-007] is restricted to VPN-only access [C3-016] with MFA enforced and confirmed to be not publicly accessible. The Customer Uploads S3 bucket [C3-004] uses pre-signed URLs for time-limited access rather than direct bucket permissions. The Pattern Library S3 bucket [C3-003] has public read blocked at the bucket policy level. GitHub [C3-008] enforces private repositories only with branch protection enabled, requiring pull request review before any production deployment. CloudFront [C3-006] serves static assets with a WAF attached.</t>
+  </si>
+  <si>
+    <t>Role-based access control in implemented and operationally enforced through Microsoft Entra ID Conditional Access rules, [C3-013]. This governs authentication and device compliance requirements for all SaaS and cloud environment access. 1Password Teams [C3-020] vaults are segmented by department, with credential access limited by function. Employee system access is provisioned per role. Devon Nakamura is noted as responsible for quarterly access reviews on privleged accounts.</t>
+  </si>
+  <si>
+    <t>Access provisioning follows the least-privilege model, by role-differentiated system access. Devon Nakamura is noted as responsible for quarterly access reviews on privleged accounts. 1Password [C3-020] vault segmentation enforces access boundaries by department. No formal access rights review is documented, no procedures for access rights are documented.</t>
+  </si>
+  <si>
+    <t>EDR coverage is not confirmed for the remaining 14 endpoints, including all MacBook Air devices assigned to Customer Success, Marketing, Operations, and Content staff. The CEO [C3-EMP-001] and CFO's [C3-EMP-002] Macbooks are not confirmed to be protected via EDR, with Confidential and Restricted data on these devices. No anti-malware or EDR solution is referenced for the standard employee device fleet. There is no evidence of a centrally managed anti-malware policy, coverage reporting, or defined response procedure for malware detection events.</t>
+  </si>
+  <si>
+    <t>PII is identified and flagged across the entire asset inventory using a dedicated 'Contains PII' column applied to all 42 assets. No formal Privacy Policy or PII handling procedure document has been identified. There is no documented process for responding to data subject access requests or right-to-erasure requests, which is a meaningful gap given C3's customer PII exposure and GDPR obligations.</t>
+  </si>
+  <si>
+    <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C3-013]. Privileged accounts are required to use hardware security keys, NIST SP 800-63B AAL3 authentication, for any admin account activity. All credentials are stored and managed by 1Password [C3-020], with vault segmentation by department, preventing cross-functional exposure.</t>
+  </si>
+  <si>
+    <t>No formal password policy is defined. No recovery procedures are defined, if Devon or Jordan lose a hardware key, there's no documented recovery path for AWS Admin or GitHub Admin access. Technical controls are in place via 1Password.</t>
+  </si>
+  <si>
+    <t>No formal documentation was found. Without a management-approved policy, the operationally enforced controls in C3-CTL-001 through C3-CTL-006 have no formal baseline to be measured against, and no ISO 27001 audit would accept technical controls without a governing policy document.</t>
+  </si>
+  <si>
+    <t>What is the specific gap you identified? Risk Consequence?</t>
   </si>
 </sst>
 </file>
@@ -1473,6 +1470,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1489,12 +1492,6 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1720,37 +1717,38 @@
   <cols>
     <col min="1" max="1" width="23.77734375" style="66" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" style="66" hidden="1" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" style="66" customWidth="1"/>
+    <col min="3" max="3" width="20.109375" style="66" customWidth="1"/>
     <col min="4" max="4" width="14" style="66" hidden="1" customWidth="1"/>
-    <col min="5" max="5" width="16.33203125" style="66" customWidth="1"/>
+    <col min="5" max="5" width="21.109375" style="66" customWidth="1"/>
     <col min="6" max="6" width="12.6640625" style="66"/>
-    <col min="7" max="7" width="45.33203125" style="66" customWidth="1"/>
+    <col min="7" max="7" width="36.33203125" style="66" customWidth="1"/>
     <col min="8" max="8" width="10.77734375" style="66" customWidth="1"/>
     <col min="9" max="11" width="12.6640625" style="66"/>
     <col min="12" max="12" width="55.109375" style="66" customWidth="1"/>
-    <col min="13" max="13" width="40.21875" style="66" customWidth="1"/>
-    <col min="14" max="14" width="24.33203125" style="66" customWidth="1"/>
-    <col min="15" max="16384" width="12.6640625" style="66"/>
+    <col min="13" max="13" width="43.21875" style="66" customWidth="1"/>
+    <col min="14" max="14" width="30.5546875" style="66" customWidth="1"/>
+    <col min="15" max="15" width="19.21875" style="66" customWidth="1"/>
+    <col min="16" max="16384" width="12.6640625" style="66"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="67"/>
-      <c r="C1" s="67"/>
-      <c r="D1" s="67"/>
-      <c r="E1" s="67"/>
-      <c r="F1" s="67"/>
-      <c r="G1" s="67"/>
-      <c r="H1" s="67"/>
-      <c r="I1" s="67"/>
-      <c r="J1" s="67"/>
-      <c r="K1" s="67"/>
-      <c r="L1" s="67"/>
-      <c r="M1" s="67"/>
-      <c r="N1" s="67"/>
-      <c r="O1" s="68"/>
+      <c r="B1" s="69"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="69"/>
+      <c r="L1" s="69"/>
+      <c r="M1" s="69"/>
+      <c r="N1" s="69"/>
+      <c r="O1" s="70"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
@@ -1764,29 +1762,29 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2" spans="1:26" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="69" t="s">
+      <c r="A2" s="71" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="67"/>
-      <c r="C2" s="67"/>
-      <c r="D2" s="67"/>
-      <c r="E2" s="68"/>
-      <c r="F2" s="70" t="s">
+      <c r="B2" s="69"/>
+      <c r="C2" s="69"/>
+      <c r="D2" s="69"/>
+      <c r="E2" s="70"/>
+      <c r="F2" s="72" t="s">
         <v>2</v>
       </c>
-      <c r="G2" s="68"/>
-      <c r="H2" s="71" t="s">
+      <c r="G2" s="70"/>
+      <c r="H2" s="73" t="s">
         <v>3</v>
       </c>
-      <c r="I2" s="67"/>
-      <c r="J2" s="67"/>
-      <c r="K2" s="67"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="72" t="s">
+      <c r="I2" s="69"/>
+      <c r="J2" s="69"/>
+      <c r="K2" s="69"/>
+      <c r="L2" s="70"/>
+      <c r="M2" s="74" t="s">
         <v>4</v>
       </c>
-      <c r="N2" s="67"/>
-      <c r="O2" s="68"/>
+      <c r="N2" s="69"/>
+      <c r="O2" s="70"/>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
       <c r="R2" s="1"/>
@@ -1895,13 +1893,13 @@
         <v>31</v>
       </c>
       <c r="M4" s="3" t="s">
+        <v>285</v>
+      </c>
+      <c r="N4" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="N4" s="3" t="s">
+      <c r="O4" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
@@ -1917,43 +1915,43 @@
     </row>
     <row r="5" spans="1:26" ht="79.8" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B5" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G5" s="5" t="s">
-        <v>41</v>
-      </c>
       <c r="H5" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J5" s="9">
         <v>2</v>
       </c>
       <c r="K5" s="58" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L5" s="62" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="M5" s="61" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="8"/>
@@ -1971,43 +1969,43 @@
     </row>
     <row r="6" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B6" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="F6" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="F6" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>47</v>
-      </c>
       <c r="H6" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I6" s="11" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J6" s="12">
         <v>2</v>
       </c>
       <c r="K6" s="59" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L6" s="63" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="M6" s="64" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="N6" s="10"/>
       <c r="O6" s="11"/>
@@ -2023,45 +2021,45 @@
       <c r="Y6" s="1"/>
       <c r="Z6" s="1"/>
     </row>
-    <row r="7" spans="1:26" ht="57" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" ht="68.400000000000006" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="D7" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="F7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>53</v>
-      </c>
       <c r="H7" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="J7" s="9">
         <v>2</v>
       </c>
       <c r="K7" s="58" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L7" s="62" t="s">
-        <v>261</v>
+        <v>282</v>
       </c>
       <c r="M7" s="61" t="s">
-        <v>262</v>
+        <v>283</v>
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="8"/>
@@ -2079,43 +2077,43 @@
     </row>
     <row r="8" spans="1:26" ht="84" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="C8" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="D8" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F8" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="H8" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I8" s="11" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J8" s="12">
         <v>2</v>
       </c>
       <c r="K8" s="59" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L8" s="63" t="s">
-        <v>259</v>
+        <v>279</v>
       </c>
       <c r="M8" s="64" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="N8" s="10"/>
       <c r="O8" s="11"/>
@@ -2133,46 +2131,46 @@
     </row>
     <row r="9" spans="1:26" ht="136.80000000000001" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="F9" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>65</v>
-      </c>
       <c r="H9" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I9" s="60" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J9" s="9">
         <v>1</v>
       </c>
       <c r="K9" s="58" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L9" s="62" t="s">
-        <v>236</v>
+        <v>277</v>
       </c>
       <c r="M9" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="N9" s="7" t="s">
         <v>235</v>
-      </c>
-      <c r="N9" s="7" t="s">
-        <v>237</v>
       </c>
       <c r="O9" s="8"/>
       <c r="P9" s="1"/>
@@ -2189,43 +2187,43 @@
     </row>
     <row r="10" spans="1:26" ht="79.8" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B10" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="C10" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="D10" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="F10" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="F10" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>71</v>
-      </c>
       <c r="H10" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I10" s="65" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J10" s="12">
         <v>2</v>
       </c>
       <c r="K10" s="59" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L10" s="63" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="M10" s="64" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="N10" s="10"/>
       <c r="O10" s="11"/>
@@ -2243,43 +2241,43 @@
     </row>
     <row r="11" spans="1:26" ht="79.8" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B11" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="C11" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="D11" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="13" t="s">
         <v>76</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="G11" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="G11" s="5" t="s">
-        <v>78</v>
-      </c>
       <c r="H11" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I11" s="60" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="J11" s="9">
         <v>1</v>
       </c>
       <c r="K11" s="58" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="L11" s="62" t="s">
-        <v>267</v>
+        <v>259</v>
       </c>
       <c r="M11" s="61" t="s">
-        <v>263</v>
+        <v>284</v>
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="8"/>
@@ -2297,43 +2295,43 @@
     </row>
     <row r="12" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="F12" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="F12" s="14" t="s">
+      <c r="G12" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="G12" s="5" t="s">
-        <v>85</v>
-      </c>
       <c r="H12" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="J12" s="12">
         <v>1</v>
       </c>
       <c r="K12" s="59" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L12" s="63" t="s">
-        <v>264</v>
+        <v>256</v>
       </c>
       <c r="M12" s="64" t="s">
-        <v>265</v>
+        <v>257</v>
       </c>
       <c r="N12" s="10"/>
       <c r="O12" s="11"/>
@@ -2351,43 +2349,43 @@
     </row>
     <row r="13" spans="1:26" ht="68.400000000000006" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="F13" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="F13" s="14" t="s">
+      <c r="G13" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="G13" s="5" t="s">
-        <v>92</v>
-      </c>
       <c r="H13" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J13" s="9">
         <v>2</v>
       </c>
       <c r="K13" s="58" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L13" s="62" t="s">
-        <v>241</v>
+        <v>281</v>
       </c>
       <c r="M13" s="61" t="s">
-        <v>266</v>
+        <v>258</v>
       </c>
       <c r="N13" s="7"/>
       <c r="O13" s="8"/>
@@ -2405,43 +2403,43 @@
     </row>
     <row r="14" spans="1:26" ht="148.19999999999999" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="F14" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="F14" s="15" t="s">
+      <c r="G14" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="G14" s="5" t="s">
-        <v>99</v>
-      </c>
       <c r="H14" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I14" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J14" s="12">
         <v>4</v>
       </c>
       <c r="K14" s="59" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L14" s="63" t="s">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="M14" s="64" t="s">
-        <v>269</v>
+        <v>261</v>
       </c>
       <c r="N14" s="10"/>
       <c r="O14" s="11"/>
@@ -2459,43 +2457,43 @@
     </row>
     <row r="15" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>102</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="F15" s="15" t="s">
+        <v>97</v>
+      </c>
+      <c r="G15" s="5" t="s">
         <v>104</v>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>105</v>
-      </c>
       <c r="H15" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I15" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J15" s="9">
         <v>2</v>
       </c>
       <c r="K15" s="58" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L15" s="62" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="M15" s="7" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="N15" s="7"/>
       <c r="O15" s="8"/>
@@ -2513,43 +2511,43 @@
     </row>
     <row r="16" spans="1:26" ht="91.2" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>106</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>107</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>108</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>109</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="F16" s="16" t="s">
         <v>110</v>
       </c>
-      <c r="F16" s="16" t="s">
+      <c r="G16" s="5" t="s">
         <v>111</v>
       </c>
-      <c r="G16" s="5" t="s">
-        <v>112</v>
-      </c>
       <c r="H16" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I16" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J16" s="12">
         <v>1</v>
       </c>
       <c r="K16" s="59" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L16" s="63" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="M16" s="64" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="N16" s="10"/>
       <c r="O16" s="11"/>
@@ -2565,45 +2563,45 @@
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
     </row>
-    <row r="17" spans="1:26" ht="114" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" ht="91.2" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>114</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>116</v>
       </c>
-      <c r="E17" s="5" t="s">
+      <c r="F17" s="16" t="s">
+        <v>110</v>
+      </c>
+      <c r="G17" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="F17" s="16" t="s">
-        <v>111</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>118</v>
-      </c>
       <c r="H17" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>243</v>
+        <v>197</v>
       </c>
       <c r="J17" s="9">
         <v>2</v>
       </c>
       <c r="K17" s="58" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="L17" s="62" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="M17" s="61" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="N17" s="7"/>
       <c r="O17" s="8"/>
@@ -2619,48 +2617,50 @@
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
     </row>
-    <row r="18" spans="1:26" ht="114" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="136.80000000000001" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>121</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>122</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="E18" s="5" t="s">
+      <c r="F18" s="17" t="s">
         <v>124</v>
       </c>
-      <c r="F18" s="17" t="s">
+      <c r="G18" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="G18" s="5" t="s">
-        <v>126</v>
-      </c>
       <c r="H18" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J18" s="9">
         <v>1</v>
       </c>
       <c r="K18" s="58" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L18" s="62" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="M18" s="61" t="s">
-        <v>272</v>
+        <v>280</v>
       </c>
       <c r="N18" s="7"/>
-      <c r="O18" s="8"/>
+      <c r="O18" s="8" t="s">
+        <v>213</v>
+      </c>
       <c r="P18" s="1"/>
       <c r="Q18" s="1"/>
       <c r="R18" s="1"/>
@@ -2673,45 +2673,45 @@
       <c r="Y18" s="1"/>
       <c r="Z18" s="1"/>
     </row>
-    <row r="19" spans="1:26" ht="114" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:26" ht="91.2" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B19" s="5" t="s">
+        <v>127</v>
+      </c>
+      <c r="C19" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="F19" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="G19" s="5" t="s">
         <v>131</v>
       </c>
-      <c r="F19" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>132</v>
-      </c>
       <c r="H19" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I19" s="11" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J19" s="12">
         <v>1</v>
       </c>
       <c r="K19" s="59" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L19" s="63" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="M19" s="64" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="N19" s="10"/>
       <c r="O19" s="11"/>
@@ -2729,43 +2729,43 @@
     </row>
     <row r="20" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B20" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="C20" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="F20" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="G20" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="F20" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>138</v>
-      </c>
       <c r="H20" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J20" s="9">
         <v>1</v>
       </c>
       <c r="K20" s="58" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L20" s="63" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="N20" s="7"/>
       <c r="O20" s="8"/>
@@ -2783,43 +2783,43 @@
     </row>
     <row r="21" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B21" s="5" t="s">
+        <v>139</v>
+      </c>
+      <c r="C21" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="E21" s="5" t="s">
         <v>142</v>
       </c>
-      <c r="E21" s="5" t="s">
+      <c r="F21" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="G21" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="F21" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>144</v>
-      </c>
       <c r="H21" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I21" s="65" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J21" s="12">
         <v>2</v>
       </c>
       <c r="K21" s="59" t="s">
-        <v>231</v>
-      </c>
-      <c r="L21" s="73" t="s">
-        <v>273</v>
+        <v>230</v>
+      </c>
+      <c r="L21" s="67" t="s">
+        <v>264</v>
       </c>
       <c r="M21" s="64" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="N21" s="10"/>
       <c r="O21" s="11"/>
@@ -2835,41 +2835,45 @@
       <c r="Y21" s="1"/>
       <c r="Z21" s="1"/>
     </row>
-    <row r="22" spans="1:26" ht="125.4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:26" ht="91.2" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B22" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C22" s="5" t="s">
         <v>146</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="E22" s="5" t="s">
+      <c r="F22" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="G22" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="F22" s="17" t="s">
-        <v>125</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>150</v>
-      </c>
       <c r="H22" s="7" t="s">
-        <v>232</v>
-      </c>
-      <c r="I22" s="8"/>
-      <c r="J22" s="9"/>
+        <v>231</v>
+      </c>
+      <c r="I22" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="J22" s="9">
+        <v>2</v>
+      </c>
       <c r="K22" s="58" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L22" s="62" t="s">
-        <v>274</v>
+        <v>265</v>
       </c>
       <c r="M22" s="61" t="s">
-        <v>275</v>
+        <v>266</v>
       </c>
       <c r="N22" s="7"/>
       <c r="O22" s="8"/>
@@ -2887,43 +2891,43 @@
     </row>
     <row r="23" spans="1:26" ht="136.80000000000001" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B23" s="5" t="s">
+        <v>152</v>
+      </c>
+      <c r="C23" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="D23" s="5" t="s">
         <v>154</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="E23" s="5" t="s">
+      <c r="F23" s="18" t="s">
         <v>156</v>
       </c>
-      <c r="F23" s="18" t="s">
+      <c r="G23" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="G23" s="5" t="s">
-        <v>158</v>
-      </c>
       <c r="H23" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I23" s="60" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="J23" s="9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K23" s="58" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L23" s="62" t="s">
-        <v>276</v>
+        <v>267</v>
       </c>
       <c r="M23" s="61" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="N23" s="7"/>
       <c r="O23" s="8"/>
@@ -2941,43 +2945,43 @@
     </row>
     <row r="24" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B24" s="5" t="s">
+        <v>159</v>
+      </c>
+      <c r="C24" s="5" t="s">
         <v>160</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>162</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="F24" s="19" t="s">
         <v>163</v>
       </c>
-      <c r="F24" s="19" t="s">
+      <c r="G24" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="G24" s="5" t="s">
-        <v>165</v>
-      </c>
       <c r="H24" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I24" s="65" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J24" s="12">
         <v>1</v>
       </c>
       <c r="K24" s="59" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="L24" s="63" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="M24" s="64" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="N24" s="10"/>
       <c r="O24" s="11"/>
@@ -2995,43 +2999,43 @@
     </row>
     <row r="25" spans="1:26" ht="102.6" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B25" s="5" t="s">
+        <v>166</v>
+      </c>
+      <c r="C25" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>162</v>
+      </c>
+      <c r="F25" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="G25" s="5" t="s">
         <v>168</v>
       </c>
-      <c r="D25" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="E25" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="F25" s="19" t="s">
-        <v>164</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>169</v>
-      </c>
       <c r="H25" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I25" s="60" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J25" s="9">
         <v>1</v>
       </c>
       <c r="K25" s="58" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="L25" s="62" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="M25" s="61" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="N25" s="7"/>
       <c r="O25" s="8"/>
@@ -3049,43 +3053,43 @@
     </row>
     <row r="26" spans="1:26" ht="125.4" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B26" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="C26" s="5" t="s">
         <v>171</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="D26" s="5" t="s">
         <v>172</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="F26" s="20" t="s">
         <v>174</v>
       </c>
-      <c r="F26" s="20" t="s">
+      <c r="G26" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="G26" s="5" t="s">
-        <v>176</v>
-      </c>
       <c r="H26" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I26" s="65" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J26" s="12">
         <v>1</v>
       </c>
       <c r="K26" s="59" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L26" s="63" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="M26" s="64" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="N26" s="10"/>
       <c r="O26" s="11"/>
@@ -3103,43 +3107,43 @@
     </row>
     <row r="27" spans="1:26" ht="148.19999999999999" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C27" s="5" t="s">
         <v>178</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="D27" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="F27" s="20" t="s">
+        <v>174</v>
+      </c>
+      <c r="G27" s="5" t="s">
         <v>181</v>
       </c>
-      <c r="F27" s="20" t="s">
-        <v>175</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>182</v>
-      </c>
       <c r="H27" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I27" s="60" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J27" s="9">
         <v>2</v>
       </c>
       <c r="K27" s="58" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L27" s="62" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="M27" s="61" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="N27" s="7"/>
       <c r="O27" s="8"/>
@@ -3157,43 +3161,43 @@
     </row>
     <row r="28" spans="1:26" ht="148.19999999999999" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B28" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="E28" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="F28" s="21" t="s">
         <v>186</v>
       </c>
-      <c r="F28" s="21" t="s">
+      <c r="G28" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="G28" s="5" t="s">
-        <v>188</v>
-      </c>
       <c r="H28" s="7" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I28" s="60" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J28" s="9">
         <v>2</v>
       </c>
       <c r="K28" s="58" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L28" s="62" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="M28" s="61" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="N28" s="7"/>
       <c r="O28" s="8"/>
@@ -3211,43 +3215,43 @@
     </row>
     <row r="29" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B29" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="D29" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="E29" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="F29" s="21" t="s">
+        <v>186</v>
+      </c>
+      <c r="G29" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="F29" s="21" t="s">
-        <v>187</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>193</v>
-      </c>
       <c r="H29" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="I29" s="11" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="J29" s="12">
         <v>4</v>
       </c>
       <c r="K29" s="59" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="L29" s="63" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="M29" s="64" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="N29" s="10"/>
       <c r="O29" s="11"/>
@@ -30309,7 +30313,7 @@
   <sheetData>
     <row r="1" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="22" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B1" s="23"/>
     </row>
@@ -30319,32 +30323,32 @@
     </row>
     <row r="3" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B3" s="27"/>
     </row>
     <row r="4" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A4" s="28" t="s">
+        <v>195</v>
+      </c>
+      <c r="B4" s="29" t="s">
         <v>196</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A5" s="30" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5" s="31" t="s">
         <v>198</v>
-      </c>
-      <c r="B5" s="31" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A6" s="32" t="s">
+        <v>199</v>
+      </c>
+      <c r="B6" s="33" t="s">
         <v>200</v>
-      </c>
-      <c r="B6" s="33" t="s">
-        <v>201</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
@@ -30353,48 +30357,48 @@
     </row>
     <row r="8" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A8" s="26" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B8" s="27"/>
     </row>
     <row r="9" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A9" s="36" t="s">
+        <v>202</v>
+      </c>
+      <c r="B9" s="37" t="s">
         <v>203</v>
-      </c>
-      <c r="B9" s="37" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A10" s="38" t="s">
+        <v>204</v>
+      </c>
+      <c r="B10" s="39" t="s">
         <v>205</v>
-      </c>
-      <c r="B10" s="39" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A11" s="40" t="s">
+        <v>206</v>
+      </c>
+      <c r="B11" s="41" t="s">
         <v>207</v>
-      </c>
-      <c r="B11" s="41" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A12" s="42" t="s">
+        <v>208</v>
+      </c>
+      <c r="B12" s="43" t="s">
         <v>209</v>
-      </c>
-      <c r="B12" s="43" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A13" s="44" t="s">
+        <v>210</v>
+      </c>
+      <c r="B13" s="45" t="s">
         <v>211</v>
-      </c>
-      <c r="B13" s="45" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
@@ -30403,32 +30407,32 @@
     </row>
     <row r="15" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A15" s="26" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B15" s="27"/>
     </row>
     <row r="16" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A16" s="46" t="s">
+        <v>213</v>
+      </c>
+      <c r="B16" s="47" t="s">
         <v>214</v>
-      </c>
-      <c r="B16" s="47" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="17" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A17" s="48" t="s">
+        <v>215</v>
+      </c>
+      <c r="B17" s="49" t="s">
         <v>216</v>
-      </c>
-      <c r="B17" s="49" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="18" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A18" s="50" t="s">
+        <v>217</v>
+      </c>
+      <c r="B18" s="51" t="s">
         <v>218</v>
-      </c>
-      <c r="B18" s="51" t="s">
-        <v>219</v>
       </c>
     </row>
     <row r="19" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
@@ -30437,32 +30441,32 @@
     </row>
     <row r="20" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A20" s="26" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B20" s="27"/>
     </row>
     <row r="21" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A21" s="52" t="s">
+        <v>220</v>
+      </c>
+      <c r="B21" s="53" t="s">
         <v>221</v>
-      </c>
-      <c r="B21" s="53" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A22" s="54" t="s">
+        <v>222</v>
+      </c>
+      <c r="B22" s="55" t="s">
         <v>223</v>
-      </c>
-      <c r="B22" s="55" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="24" x14ac:dyDescent="0.25">
       <c r="A23" s="56" t="s">
+        <v>224</v>
+      </c>
+      <c r="B23" s="57" t="s">
         <v>225</v>
-      </c>
-      <c r="B23" s="57" t="s">
-        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="13.2" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Ok Gap Descrip in more professional language
</commit_message>
<xml_diff>
--- a/compliance/Control_Matrix_Mapping.xlsx
+++ b/compliance/Control_Matrix_Mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kate\OneDrive\Documents\GRC_Risk_Assessment\C3-GRC\compliance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EDA40CE-F714-4E1E-BF25-9B052CD94C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ECC0592-3037-4134-AD36-B7CB7C96A9A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Control Matrix Mapping" sheetId="1" r:id="rId1"/>
@@ -744,25 +744,16 @@
     <t xml:space="preserve">Partial </t>
   </si>
   <si>
-    <t>There is no formal access control policy.</t>
-  </si>
-  <si>
     <t>Develop a formal access control policy.</t>
   </si>
   <si>
     <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C3-013]. Privileged accounts are required to use hardware security keys for any admin account activity. GitHub SSO [C3-008] and 1Password SSO [C3-020] are enforced via Entra ID, preventing local credential bypass. AWS IAM is federated via SAML from Entra ID [C3-013], meaning Entra ID governs authentication even for cloud resource access.</t>
   </si>
   <si>
-    <t>No formal authentication standard or Privileged Access Management (PAM) policy document has been identified. Secure authentication is technically enforced but not formally governed by a written standard communicated to all staff.</t>
-  </si>
-  <si>
     <t xml:space="preserve">Missing </t>
   </si>
   <si>
     <t>No security awareness training program has been identified. There is no reference to a training platform, completion tracking mechanism, training schedule, or role-based curriculum for any of C3's 16 employees. MFA and hardware key requirements are technically enforced at the tooling level, indicating some baseline security hygiene exists operationally. However, there is no evidence that staff have received formal instruction on phishing recognition, incident reporting, acceptable use, data handling, or any other security awareness topic.</t>
-  </si>
-  <si>
-    <t>No formal classification policy or labeling standard has been identified defining each tier's handling requirements or mandating consistent labeling on documents and files outside of the asset inventory context.</t>
   </si>
   <si>
     <t>Jordan Ellis [DevOps &amp; Cloud Engineer, EMP-006] is identified as the Infrastructure-as-Code (IaC) owner, with all AWS infrastructure managed through IaC stored in the GitHub organization [C3-008]. GitHub Actions [C3-009) automates deployment pipelines and enforces consistent deployment processes, reducing manual configuration drift. Branch protection on GitHub requires pull request review before any infrastructure code change is applied, providing a change control mechanism. Microsoft Intune MDM [C3-010] manages endpoint configuration baselines for all 17 devices. Entra ID Conditional Access [C3-013] enforces compliant device requirements, acting as a soft configuration baseline gate.</t>
@@ -807,13 +798,7 @@
     <t>No formal log management policy has been identified defining required log sources, minimum retention periods per asset class, log integrity requirements, or procedures for log review and investigation. No centralized SIEM aggregating logs across SaaS, endpoints, and cloud has been identified.</t>
   </si>
   <si>
-    <t>Technical controls are in place via 1Password, however, no formal access rights review schedule, documented provisioning and deprovisioning procedures, or periodic recertification process have been identified beyond the noted quarterly review for privileged accounts.</t>
-  </si>
-  <si>
     <t>C3 operates in a regulatory environment touching multiple frameworks. PCI DSS obligations arise from subscription payment processing via Stripe [C3-012]; C3 mitigates direct PCI scope by tokenizing all payment card data through Stripe rather than storing raw card data. ISO 27001 compliance tags are applied to all 42 assets in the asset inventory. Customer PII and employee PII are present across multiple assets [C3-001, C3-002, C3-004, C3-015, C3-024], indicating GDPR and applicable U.S. privacy law obligations. Marcus Okafor is noted as responsible for finance and compliance-adjacent functions.</t>
-  </si>
-  <si>
-    <t>Regulatory awareness appears operationally embedded but not formally catalogued or reviewed on a defined schedule. No formal legal and regulatory register has been identified documenting all applicable obligations, their sources, review dates, or responsible owners.</t>
   </si>
   <si>
     <t>No formal Privacy Policy or PII handling procedure document has been identified. There is no documented process for responding to data subject access requests or right-to-erasure requests.</t>
@@ -823,9 +808,6 @@
   </si>
   <si>
     <t>C3 maintains a formal asset inventory covering 42 assets across five categories: cloud infrastructure [servers, databases, storage, networking), SaaS tools, identity and access management, payment processing, and employee endpoints. Each asset record includes Asset ID, Friendly Name, Asset Type, Asset Category, Business Owner, Technical Owner, Department, Custodian, Environment, Data Classification, Data Types Stored, PII and PCI flags, Sensitivity Score (1-5), ISO 27001 scope flag, Compliance Tags, Status, Date Added, and Last Updated. Asset IDs follow a consistent naming convention (C3-001 through C3-025 for infrastructure/SaaS; C3-EMP-001 through C3-EMP-016B for endpoints). One decommissioned asset (C3-017, Zoom, closed January 2025) is retained in the inventory with decommission date recorded. The inventory is actively maintained and comprehensive.</t>
-  </si>
-  <si>
-    <t>The formal asset inventory appears to be an accurate, living document, however, there is no formal procedure or policy outlining updating the inventory.</t>
   </si>
   <si>
     <t xml:space="preserve">Information classification is applied to all 42 assets in the asset inventory using a four-tier scheme: Restricted, Confidential, Internal, and Public. No assets are currently classified Public. Classification is recorded in a dedicated 'Data Classification' column for every asset. Restricted assets include the Production Database [C3-002], Admin Portal [C3-007], Stripe account [C3-012], Entra ID [C3-013], 1Password [C3-020], Rippling [C3-024], and QuickBooks [C3-025], all carrying sensitivity scores of 4 or 5. A supplementary 'Sensitivity Score (1-5)' column provides a numeric risk weighting alongside the classification label. Data types stored are documented per asset to support classification decisions. </t>
@@ -844,12 +826,6 @@
   </si>
   <si>
     <t>All 17 employee endpoints are enrolled in Microsoft Intune MDM via the M365 E3 tenant [C3-010], which enforces device compliance as a prerequisite for Entra ID Conditional Access. FileVault full-disk encryption is confirmed on all 16 MacBook devices. The iPad Pro [C3-EMP-016B] is enrolled under iPadOS 17.3. EDR is deployed on three high-risk MacBook Pros (CTO, DevOps Engineer, Senior Software Engineer). Hardware security keys are enforced on all admin-level devices. OS versions are consistent across the Mac fleet (macOS Sonoma 14.4). EDR coverage is confirmed for only 3 of 17 endpoints. No formal endpoint security policy or acceptable use policy has been identified. Screen lock enforcement is confirmed only on the CEO device (2 minutes); uniform enforcement across all 17 devices is not individually verified in the asset inventory.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No formal policy is identified or referenced. The control is operationally practiced, but not formally documented or communicated as a policy artifact. </t>
-  </si>
-  <si>
-    <t>The control is operationally practiced, but not formally documented or communicated as a policy artifact. The process appears to be operationally managed through Rippling and Entra ID but without a documented runbook defining steps, timelines, or verification requirements for provisioning and deprovisioning.</t>
   </si>
   <si>
     <t>There is no security awareness training program. There is no evidence that staff have received formal instruction on phishing recognition, incident reporting, acceptable use, data handling, or any other security awareness topic.</t>
@@ -891,13 +867,37 @@
     <t>All 16 employees are enrolled in MFA, enforced by Entra ID Conditional Access [C3-013]. Privileged accounts are required to use hardware security keys, NIST SP 800-63B AAL3 authentication, for any admin account activity. All credentials are stored and managed by 1Password [C3-020], with vault segmentation by department, preventing cross-functional exposure.</t>
   </si>
   <si>
-    <t>No formal password policy is defined. No recovery procedures are defined, if Devon or Jordan lose a hardware key, there's no documented recovery path for AWS Admin or GitHub Admin access. Technical controls are in place via 1Password.</t>
+    <t>What is the specific gap you identified? Risk Consequence?</t>
   </si>
   <si>
-    <t>No formal documentation was found. Without a management-approved policy, the operationally enforced controls in C3-CTL-001 through C3-CTL-006 have no formal baseline to be measured against, and no ISO 27001 audit would accept technical controls without a governing policy document.</t>
+    <t>The absence of a formal access control policy results in inconsistent access provisioning and increases the risk of unauthorized access.</t>
   </si>
   <si>
-    <t>What is the specific gap you identified? Risk Consequence?</t>
+    <t>While the control appears to be operationally performed, it is not formally documented or standardized, reducing consistency and limiting auditability.</t>
+  </si>
+  <si>
+    <t>There is no formally defined password or credential recovery policy, increasing the risk of weak authentication practices and unauthorized access.</t>
+  </si>
+  <si>
+    <t>Technical controls (e.g., password management tools) are in place; however, the absence of a formal policy or governance framework may result in inconsistent usage and enforcement.</t>
+  </si>
+  <si>
+    <t>The absence of a formal access control policy results in undefined access requirements and increases the risk of inappropriate or unauthorized access.</t>
+  </si>
+  <si>
+    <t>There is no formally established authentication or privileged access standard, leading to inconsistent implementation and elevated risk of unauthorized privilege escalation.</t>
+  </si>
+  <si>
+    <t>No formal documentation was identified; as a result, control execution may vary and cannot be consistently validated or audited.</t>
+  </si>
+  <si>
+    <t>There is no formal Privacy Policy or defined procedures for handling PII, increasing the risk of non-compliance with data protection regulations.</t>
+  </si>
+  <si>
+    <t>The asset inventory appears incomplete or informal, limiting visibility into managed assets and increasing the risk of unmanaged or unprotected resources.</t>
+  </si>
+  <si>
+    <t>No formal classification policy or labeling standard has been identified; increasing the risk of mishandling sensitive information.</t>
   </si>
 </sst>
 </file>
@@ -1893,7 +1893,7 @@
         <v>31</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="N4" s="3" t="s">
         <v>32</v>
@@ -1948,10 +1948,10 @@
         <v>226</v>
       </c>
       <c r="L5" s="62" t="s">
-        <v>278</v>
+        <v>270</v>
       </c>
       <c r="M5" s="61" t="s">
-        <v>268</v>
+        <v>276</v>
       </c>
       <c r="N5" s="7"/>
       <c r="O5" s="8"/>
@@ -2005,7 +2005,7 @@
         <v>232</v>
       </c>
       <c r="M6" s="64" t="s">
-        <v>269</v>
+        <v>277</v>
       </c>
       <c r="N6" s="10"/>
       <c r="O6" s="11"/>
@@ -2056,10 +2056,10 @@
         <v>226</v>
       </c>
       <c r="L7" s="62" t="s">
-        <v>282</v>
+        <v>274</v>
       </c>
       <c r="M7" s="61" t="s">
-        <v>283</v>
+        <v>278</v>
       </c>
       <c r="N7" s="7"/>
       <c r="O7" s="8"/>
@@ -2110,10 +2110,10 @@
         <v>226</v>
       </c>
       <c r="L8" s="63" t="s">
+        <v>271</v>
+      </c>
+      <c r="M8" s="64" t="s">
         <v>279</v>
-      </c>
-      <c r="M8" s="64" t="s">
-        <v>255</v>
       </c>
       <c r="N8" s="10"/>
       <c r="O8" s="11"/>
@@ -2164,13 +2164,13 @@
         <v>226</v>
       </c>
       <c r="L9" s="62" t="s">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="M9" s="7" t="s">
+        <v>280</v>
+      </c>
+      <c r="N9" s="7" t="s">
         <v>234</v>
-      </c>
-      <c r="N9" s="7" t="s">
-        <v>235</v>
       </c>
       <c r="O9" s="8"/>
       <c r="P9" s="1"/>
@@ -2220,10 +2220,10 @@
         <v>226</v>
       </c>
       <c r="L10" s="63" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="M10" s="64" t="s">
-        <v>237</v>
+        <v>281</v>
       </c>
       <c r="N10" s="10"/>
       <c r="O10" s="11"/>
@@ -2265,7 +2265,7 @@
         <v>231</v>
       </c>
       <c r="I11" s="60" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="J11" s="9">
         <v>1</v>
@@ -2274,10 +2274,10 @@
         <v>228</v>
       </c>
       <c r="L11" s="62" t="s">
-        <v>259</v>
+        <v>254</v>
       </c>
       <c r="M11" s="61" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="N11" s="7"/>
       <c r="O11" s="8"/>
@@ -2319,7 +2319,7 @@
         <v>231</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="J12" s="12">
         <v>1</v>
@@ -2328,10 +2328,10 @@
         <v>229</v>
       </c>
       <c r="L12" s="63" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="M12" s="64" t="s">
-        <v>257</v>
+        <v>283</v>
       </c>
       <c r="N12" s="10"/>
       <c r="O12" s="11"/>
@@ -2382,10 +2382,10 @@
         <v>229</v>
       </c>
       <c r="L13" s="62" t="s">
-        <v>281</v>
+        <v>273</v>
       </c>
       <c r="M13" s="61" t="s">
-        <v>258</v>
+        <v>253</v>
       </c>
       <c r="N13" s="7"/>
       <c r="O13" s="8"/>
@@ -2436,10 +2436,10 @@
         <v>230</v>
       </c>
       <c r="L14" s="63" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="M14" s="64" t="s">
-        <v>261</v>
+        <v>284</v>
       </c>
       <c r="N14" s="10"/>
       <c r="O14" s="11"/>
@@ -2490,10 +2490,10 @@
         <v>229</v>
       </c>
       <c r="L15" s="62" t="s">
-        <v>262</v>
-      </c>
-      <c r="M15" s="7" t="s">
-        <v>240</v>
+        <v>256</v>
+      </c>
+      <c r="M15" s="61" t="s">
+        <v>285</v>
       </c>
       <c r="N15" s="7"/>
       <c r="O15" s="8"/>
@@ -2544,10 +2544,10 @@
         <v>227</v>
       </c>
       <c r="L16" s="63" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="M16" s="64" t="s">
-        <v>270</v>
+        <v>262</v>
       </c>
       <c r="N16" s="10"/>
       <c r="O16" s="11"/>
@@ -2563,7 +2563,7 @@
       <c r="Y16" s="1"/>
       <c r="Z16" s="1"/>
     </row>
-    <row r="17" spans="1:26" ht="91.2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:26" ht="79.8" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>112</v>
       </c>
@@ -2598,10 +2598,10 @@
         <v>227</v>
       </c>
       <c r="L17" s="62" t="s">
-        <v>271</v>
+        <v>263</v>
       </c>
       <c r="M17" s="61" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="N17" s="7"/>
       <c r="O17" s="8"/>
@@ -2617,7 +2617,7 @@
       <c r="Y17" s="1"/>
       <c r="Z17" s="1"/>
     </row>
-    <row r="18" spans="1:26" ht="136.80000000000001" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:26" ht="125.4" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>118</v>
       </c>
@@ -2652,10 +2652,10 @@
         <v>230</v>
       </c>
       <c r="L18" s="62" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="M18" s="61" t="s">
-        <v>280</v>
+        <v>272</v>
       </c>
       <c r="N18" s="7"/>
       <c r="O18" s="8" t="s">
@@ -2708,10 +2708,10 @@
         <v>226</v>
       </c>
       <c r="L19" s="63" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="M19" s="64" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="N19" s="10"/>
       <c r="O19" s="11"/>
@@ -2762,10 +2762,10 @@
         <v>230</v>
       </c>
       <c r="L20" s="63" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="M20" s="7" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="N20" s="7"/>
       <c r="O20" s="8"/>
@@ -2816,10 +2816,10 @@
         <v>230</v>
       </c>
       <c r="L21" s="67" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="M21" s="64" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="N21" s="10"/>
       <c r="O21" s="11"/>
@@ -2870,10 +2870,10 @@
         <v>230</v>
       </c>
       <c r="L22" s="62" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="M22" s="61" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="N22" s="7"/>
       <c r="O22" s="8"/>
@@ -2924,10 +2924,10 @@
         <v>230</v>
       </c>
       <c r="L23" s="62" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="M23" s="61" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="N23" s="7"/>
       <c r="O23" s="8"/>
@@ -2978,10 +2978,10 @@
         <v>229</v>
       </c>
       <c r="L24" s="63" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="M24" s="64" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="N24" s="10"/>
       <c r="O24" s="11"/>
@@ -3032,10 +3032,10 @@
         <v>230</v>
       </c>
       <c r="L25" s="62" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="M25" s="61" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="N25" s="7"/>
       <c r="O25" s="8"/>
@@ -3051,7 +3051,7 @@
       <c r="Y25" s="1"/>
       <c r="Z25" s="1"/>
     </row>
-    <row r="26" spans="1:26" ht="125.4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:26" ht="114" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>158</v>
       </c>
@@ -3086,10 +3086,10 @@
         <v>226</v>
       </c>
       <c r="L26" s="63" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="M26" s="64" t="s">
-        <v>273</v>
+        <v>265</v>
       </c>
       <c r="N26" s="10"/>
       <c r="O26" s="11"/>
@@ -3140,10 +3140,10 @@
         <v>226</v>
       </c>
       <c r="L27" s="62" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="M27" s="61" t="s">
-        <v>274</v>
+        <v>266</v>
       </c>
       <c r="N27" s="7"/>
       <c r="O27" s="8"/>
@@ -3159,7 +3159,7 @@
       <c r="Y27" s="1"/>
       <c r="Z27" s="1"/>
     </row>
-    <row r="28" spans="1:26" ht="148.19999999999999" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:26" ht="159.6" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
         <v>169</v>
       </c>
@@ -3194,10 +3194,10 @@
         <v>226</v>
       </c>
       <c r="L28" s="62" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="M28" s="61" t="s">
-        <v>275</v>
+        <v>267</v>
       </c>
       <c r="N28" s="7"/>
       <c r="O28" s="8"/>
@@ -3213,7 +3213,7 @@
       <c r="Y28" s="1"/>
       <c r="Z28" s="1"/>
     </row>
-    <row r="29" spans="1:26" ht="114" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:26" ht="125.4" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
         <v>176</v>
       </c>
@@ -3248,10 +3248,10 @@
         <v>226</v>
       </c>
       <c r="L29" s="63" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="M29" s="64" t="s">
-        <v>276</v>
+        <v>268</v>
       </c>
       <c r="N29" s="10"/>
       <c r="O29" s="11"/>

</xml_diff>